<commit_message>
Ignore standalone assembly_designer package repo; update regenerated example outputs and packaging metadata
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/03 Sequencing/02 From folder/alignment_results.xlsx
+++ b/examples/03 Sequencing/02 From folder/alignment_results.xlsx
@@ -73,411 +73,411 @@
     <t>suspicious</t>
   </si>
   <si>
+    <t>EF73802034_EF73802034</t>
+  </si>
+  <si>
+    <t>EF73802045_EF73802045</t>
+  </si>
+  <si>
+    <t>EF73802035_EF73802035</t>
+  </si>
+  <si>
+    <t>EF73802038_EF73802038</t>
+  </si>
+  <si>
+    <t>EF73802047_EF73802047</t>
+  </si>
+  <si>
     <t>EF73802036_EF73802036</t>
   </si>
   <si>
-    <t>EF73802038_EF73802038</t>
-  </si>
-  <si>
-    <t>EF73802045_EF73802045</t>
+    <t>EF73802046_EF73802046</t>
   </si>
   <si>
     <t>EF73802033_EF73802033</t>
   </si>
   <si>
-    <t>EF73802034_EF73802034</t>
+    <t>EF73802057_EF73802057</t>
+  </si>
+  <si>
+    <t>EF73802048_EF73802048</t>
   </si>
   <si>
     <t>EF73802037_EF73802037</t>
   </si>
   <si>
-    <t>EF73802046_EF73802046</t>
-  </si>
-  <si>
-    <t>EF73802035_EF73802035</t>
+    <t>EF73802059_EF73802059</t>
   </si>
   <si>
     <t>EF73802049_EF73802049</t>
   </si>
   <si>
-    <t>EF73802057_EF73802057</t>
-  </si>
-  <si>
-    <t>EF73802047_EF73802047</t>
-  </si>
-  <si>
-    <t>EF73802048_EF73802048</t>
+    <t>EF73802060_EF73802060</t>
+  </si>
+  <si>
+    <t>EF73802058_EF73802058</t>
+  </si>
+  <si>
+    <t>EF73802070_EF73802070</t>
+  </si>
+  <si>
+    <t>EF73802069_EF73802069</t>
   </si>
   <si>
     <t>EF73802050_EF73802050</t>
   </si>
   <si>
-    <t>EF73802060_EF73802060</t>
-  </si>
-  <si>
-    <t>EF73802059_EF73802059</t>
-  </si>
-  <si>
-    <t>EF73802069_EF73802069</t>
-  </si>
-  <si>
-    <t>EF73802058_EF73802058</t>
+    <t>EF73802061_EF73802061</t>
+  </si>
+  <si>
+    <t>EF73802072_EF73802072</t>
   </si>
   <si>
     <t>EF73802071_EF73802071</t>
   </si>
   <si>
-    <t>EF73802070_EF73802070</t>
-  </si>
-  <si>
-    <t>EF73802061_EF73802061</t>
-  </si>
-  <si>
     <t>EF73802073_EF73802073</t>
   </si>
   <si>
-    <t>EF73802072_EF73802072</t>
+    <t>EF73802093_EF73802093</t>
+  </si>
+  <si>
+    <t>EF73802081_EF73802081</t>
   </si>
   <si>
     <t>EF73802082_EF73802082</t>
   </si>
   <si>
+    <t>EF73802094_EF73802094</t>
+  </si>
+  <si>
     <t>EF73802085_EF73802085</t>
   </si>
   <si>
-    <t>EF73802081_EF73802081</t>
+    <t>EF73802083_EF73802083</t>
   </si>
   <si>
     <t>EF73802084_EF73802084</t>
   </si>
   <si>
-    <t>EF73802093_EF73802093</t>
+    <t>EF73802106_EF73802106</t>
   </si>
   <si>
     <t>EF73802095_EF73802095</t>
   </si>
   <si>
-    <t>EF73802094_EF73802094</t>
-  </si>
-  <si>
-    <t>EF73802083_EF73802083</t>
+    <t>EF73802108_EF73802108</t>
+  </si>
+  <si>
+    <t>EF73802096_EF73802096</t>
   </si>
   <si>
     <t>EF73802105_EF73802105</t>
   </si>
   <si>
-    <t>EF73802108_EF73802108</t>
+    <t>EF73802129_EF73802129</t>
+  </si>
+  <si>
+    <t>EF73802109_EF73802109</t>
+  </si>
+  <si>
+    <t>EF73802130_EF73802130</t>
   </si>
   <si>
     <t>EF73802107_EF73802107</t>
   </si>
   <si>
-    <t>EF73802106_EF73802106</t>
-  </si>
-  <si>
-    <t>EF73802109_EF73802109</t>
-  </si>
-  <si>
-    <t>EF73802129_EF73802129</t>
+    <t>EF73802133_EF73802133</t>
   </si>
   <si>
     <t>EF73802131_EF73802131</t>
   </si>
   <si>
-    <t>EF73802096_EF73802096</t>
-  </si>
-  <si>
     <t>EF73802132_EF73802132</t>
   </si>
   <si>
-    <t>EF73802130_EF73802130</t>
-  </si>
-  <si>
-    <t>EF73802133_EF73802133</t>
+    <t>J23100_AB_B0033m_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
+  </si>
+  <si>
+    <t>J23100_AB_BCD12_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
+  </si>
+  <si>
+    <t>J23103_AB_BCD8_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
+  </si>
+  <si>
+    <t>R0010_AB_B0032m_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
+  </si>
+  <si>
+    <t>J23106_AB_BCD8_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
   </si>
   <si>
     <t>J23106_AB_B0033m_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
   </si>
   <si>
-    <t>R0010_AB_B0032m_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
-  </si>
-  <si>
-    <t>J23100_AB_BCD12_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
+    <t>J23103_AB_B0033m_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
   </si>
   <si>
     <t>J23102_AB_BCD12_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
   </si>
   <si>
-    <t>J23100_AB_B0033m_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
+    <t>J23103_AB_BCD12_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
+  </si>
+  <si>
+    <t>J23107_AB_B0033m_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
   </si>
   <si>
     <t>J23107_AB_B0034m_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
   </si>
   <si>
-    <t>J23103_AB_B0033m_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
-  </si>
-  <si>
-    <t>J23103_AB_BCD8_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
+    <t>J23107_AB_BCD8_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
   </si>
   <si>
     <t>J23116_AB_B0034m_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
   </si>
   <si>
-    <t>J23103_AB_BCD12_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
-  </si>
-  <si>
-    <t>J23106_AB_BCD8_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
-  </si>
-  <si>
-    <t>J23107_AB_B0033m_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
-  </si>
-  <si>
     <t>J23116_AB_B0033m_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
   </si>
   <si>
-    <t>J23107_AB_BCD8_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
-  </si>
-  <si>
     <t>J23106_AB_BCD12_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
   </si>
   <si>
+    <t>R0010_AB_B0034m_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
+  </si>
+  <si>
+    <t>R0010_AB_B0033m_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
+  </si>
+  <si>
     <t>J23116_AB_BCD8_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
   </si>
   <si>
-    <t>R0010_AB_B0034m_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
-  </si>
-  <si>
     <t>J23102_AB_B0032m_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
   </si>
   <si>
-    <t>R0010_AB_B0033m_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
+    <t>J23116_AB_BCD12_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
+  </si>
+  <si>
+    <t>J23107_AB_BCD12_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
   </si>
   <si>
     <t>J23100_AB_B0032m_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
   </si>
   <si>
-    <t>J23107_AB_BCD12_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
+    <t>R0010_AB_BCD8_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
   </si>
   <si>
     <t>J23102_AB_B0034m_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
   </si>
   <si>
-    <t>J23116_AB_BCD12_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
-  </si>
-  <si>
-    <t>R0010_AB_BCD8_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
+    <t>J23102_AB_BCD8_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
+  </si>
+  <si>
+    <t>J23103_AB_B0034m_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
+  </si>
+  <si>
+    <t>J23100_AB_B0034m_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
   </si>
   <si>
     <t>R0010_AB_BCD12_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
   </si>
   <si>
-    <t>J23103_AB_B0034m_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
-  </si>
-  <si>
-    <t>J23102_AB_BCD8_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
+    <t>J23102_AB_B0033m_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
   </si>
   <si>
     <t>J23106_AB_B0032m_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
   </si>
   <si>
-    <t>J23102_AB_B0033m_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
-  </si>
-  <si>
-    <t>J23100_AB_B0034m_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
-  </si>
-  <si>
     <t>J23106_AB_B0034m_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
   </si>
   <si>
     <t>J23107_AB_B0032m_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
   </si>
   <si>
+    <t>J23100_AB_B0033m_BC_</t>
+  </si>
+  <si>
+    <t>J23100_AB_BCD12_BC_D</t>
+  </si>
+  <si>
+    <t>J23103_AB_BCD8_BC_DV</t>
+  </si>
+  <si>
+    <t>R0010_AB_B0032m_BC_D</t>
+  </si>
+  <si>
+    <t>J23106_AB_BCD8_BC_DV</t>
+  </si>
+  <si>
     <t>J23106_AB_B0033m_BC_</t>
   </si>
   <si>
-    <t>R0010_AB_B0032m_BC_D</t>
-  </si>
-  <si>
-    <t>J23100_AB_BCD12_BC_D</t>
+    <t>J23103_AB_B0033m_BC_</t>
   </si>
   <si>
     <t>J23102_AB_BCD12_BC_D</t>
   </si>
   <si>
-    <t>J23100_AB_B0033m_BC_</t>
+    <t>J23103_AB_BCD12_BC_D</t>
+  </si>
+  <si>
+    <t>J23107_AB_B0033m_BC_</t>
   </si>
   <si>
     <t>J23107_AB_B0034m_BC_</t>
   </si>
   <si>
-    <t>J23103_AB_B0033m_BC_</t>
-  </si>
-  <si>
-    <t>J23103_AB_BCD8_BC_DV</t>
+    <t>J23107_AB_BCD8_BC_DV</t>
   </si>
   <si>
     <t>J23116_AB_B0034m_BC_</t>
   </si>
   <si>
-    <t>J23103_AB_BCD12_BC_D</t>
-  </si>
-  <si>
-    <t>J23106_AB_BCD8_BC_DV</t>
-  </si>
-  <si>
-    <t>J23107_AB_B0033m_BC_</t>
-  </si>
-  <si>
     <t>J23116_AB_B0033m_BC_</t>
   </si>
   <si>
-    <t>J23107_AB_BCD8_BC_DV</t>
-  </si>
-  <si>
     <t>J23106_AB_BCD12_BC_D</t>
   </si>
   <si>
+    <t>R0010_AB_B0034m_BC_D</t>
+  </si>
+  <si>
+    <t>R0010_AB_B0033m_BC_D</t>
+  </si>
+  <si>
     <t>J23116_AB_BCD8_BC_DV</t>
   </si>
   <si>
-    <t>R0010_AB_B0034m_BC_D</t>
-  </si>
-  <si>
     <t>J23102_AB_B0032m_BC_</t>
   </si>
   <si>
-    <t>R0010_AB_B0033m_BC_D</t>
+    <t>J23116_AB_BCD12_BC_D</t>
+  </si>
+  <si>
+    <t>J23107_AB_BCD12_BC_D</t>
   </si>
   <si>
     <t>J23100_AB_B0032m_BC_</t>
   </si>
   <si>
-    <t>J23107_AB_BCD12_BC_D</t>
+    <t>R0010_AB_BCD8_BC_DVA</t>
   </si>
   <si>
     <t>J23102_AB_B0034m_BC_</t>
   </si>
   <si>
-    <t>J23116_AB_BCD12_BC_D</t>
-  </si>
-  <si>
-    <t>R0010_AB_BCD8_BC_DVA</t>
+    <t>J23102_AB_BCD8_BC_DV</t>
+  </si>
+  <si>
+    <t>J23103_AB_B0034m_BC_</t>
+  </si>
+  <si>
+    <t>J23100_AB_B0034m_BC_</t>
   </si>
   <si>
     <t>R0010_AB_BCD12_BC_DV</t>
   </si>
   <si>
-    <t>J23103_AB_B0034m_BC_</t>
-  </si>
-  <si>
-    <t>J23102_AB_BCD8_BC_DV</t>
+    <t>J23102_AB_B0033m_BC_</t>
   </si>
   <si>
     <t>J23106_AB_B0032m_BC_</t>
   </si>
   <si>
-    <t>J23102_AB_B0033m_BC_</t>
-  </si>
-  <si>
-    <t>J23100_AB_B0034m_BC_</t>
-  </si>
-  <si>
     <t>J23106_AB_B0034m_BC_</t>
   </si>
   <si>
     <t>J23107_AB_B0032m_BC_</t>
   </si>
   <si>
+    <t>J23100_B0033m_ecPanD_B0015</t>
+  </si>
+  <si>
+    <t>J23100_BCD12_ecPanD_B0015</t>
+  </si>
+  <si>
+    <t>J23103_BCD8_ecPanD_B0015</t>
+  </si>
+  <si>
+    <t>B0032m_ecPanD_B0015</t>
+  </si>
+  <si>
+    <t>J23106_BCD8_ecPanD_B0015</t>
+  </si>
+  <si>
     <t>J23106_B0033m_ecPanD_B0015</t>
   </si>
   <si>
-    <t>B0032m_ecPanD_B0015</t>
-  </si>
-  <si>
-    <t>J23100_BCD12_ecPanD_B0015</t>
+    <t>J23103_B0033m_ecPanD_B0015</t>
   </si>
   <si>
     <t>J23102_BCD12_ecPanD_B0015</t>
   </si>
   <si>
-    <t>J23100_B0033m_ecPanD_B0015</t>
+    <t>J23103_BCD12_ecPanD_B0015</t>
+  </si>
+  <si>
+    <t>J23107_B0033m_ecPanD_B0015</t>
   </si>
   <si>
     <t>J23107_B0034m_ecPanD_B0015</t>
   </si>
   <si>
-    <t>J23103_B0033m_ecPanD_B0015</t>
-  </si>
-  <si>
-    <t>J23103_BCD8_ecPanD_B0015</t>
+    <t>J23107_BCD8_ecPanD_B0015</t>
   </si>
   <si>
     <t>J23116_B0034m_ecPanD_B0015</t>
   </si>
   <si>
-    <t>J23103_BCD12_ecPanD_B0015</t>
-  </si>
-  <si>
-    <t>J23106_BCD8_ecPanD_B0015</t>
-  </si>
-  <si>
-    <t>J23107_B0033m_ecPanD_B0015</t>
-  </si>
-  <si>
     <t>J23116_B0033m_ecPanD_B0015</t>
   </si>
   <si>
-    <t>J23107_BCD8_ecPanD_B0015</t>
-  </si>
-  <si>
     <t>J23106_BCD12_ecPanD_B0015</t>
   </si>
   <si>
+    <t>B0034m_ecPanD_B0015</t>
+  </si>
+  <si>
+    <t>B0033m_ecPanD_B0015</t>
+  </si>
+  <si>
     <t>J23116_BCD8_ecPanD_B0015</t>
   </si>
   <si>
-    <t>B0034m_ecPanD_B0015</t>
-  </si>
-  <si>
     <t>J23102_B0032m_ecPanD_B0015</t>
   </si>
   <si>
-    <t>B0033m_ecPanD_B0015</t>
+    <t>J23116_BCD12_ecPanD_B0015</t>
+  </si>
+  <si>
+    <t>J23107_BCD12_ecPanD_B0015</t>
   </si>
   <si>
     <t>J23100_B0032m_ecPanD_B0015</t>
   </si>
   <si>
-    <t>J23107_BCD12_ecPanD_B0015</t>
+    <t>BCD8_ecPanD_B0015</t>
   </si>
   <si>
     <t>J23102_B0034m_ecPanD_B0015</t>
   </si>
   <si>
-    <t>J23116_BCD12_ecPanD_B0015</t>
-  </si>
-  <si>
-    <t>BCD8_ecPanD_B0015</t>
+    <t>J23102_BCD8_ecPanD_B0015</t>
+  </si>
+  <si>
+    <t>J23103_B0034m_ecPanD_B0015</t>
+  </si>
+  <si>
+    <t>J23100_B0034m_ecPanD_B0015</t>
   </si>
   <si>
     <t>BCD12_ecPanD_B0015</t>
   </si>
   <si>
-    <t>J23103_B0034m_ecPanD_B0015</t>
-  </si>
-  <si>
-    <t>J23102_BCD8_ecPanD_B0015</t>
+    <t>J23102_B0033m_ecPanD_B0015</t>
   </si>
   <si>
     <t>J23106_B0032m_ecPanD_B0015</t>
   </si>
   <si>
-    <t>J23102_B0033m_ecPanD_B0015</t>
-  </si>
-  <si>
-    <t>J23100_B0034m_ecPanD_B0015</t>
-  </si>
-  <si>
     <t>J23106_B0034m_ecPanD_B0015</t>
   </si>
   <si>
@@ -487,99 +487,99 @@
     <t>F</t>
   </si>
   <si>
+    <t>promoter:J23100 (100%), 5'UTR:B0033m (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
+  </si>
+  <si>
+    <t>promoter:J23100 (100%), 5'UTR:BCD12 (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
+  </si>
+  <si>
+    <t>promoter:J23103 (100%), 5'UTR:BCD8 (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
+  </si>
+  <si>
+    <t>promoter:R0010 (100%), 5'UTR:B0032m (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
+  </si>
+  <si>
+    <t>promoter:J23106 (100%), 5'UTR:BCD8 (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
+  </si>
+  <si>
     <t>promoter:J23106 (100%), 5'UTR:B0033m (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
   </si>
   <si>
-    <t>promoter:R0010 (100%), 5'UTR:B0032m (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
-  </si>
-  <si>
-    <t>promoter:J23100 (100%), 5'UTR:BCD12 (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
+    <t>promoter:J23103 (100%), 5'UTR:B0033m (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
   </si>
   <si>
     <t>promoter:J23102 (100%), 5'UTR:BCD12 (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
   </si>
   <si>
-    <t>promoter:J23100 (100%), 5'UTR:B0033m (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
+    <t>promoter:J23103 (100%), 5'UTR:BCD12 (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
+  </si>
+  <si>
+    <t>promoter:J23107 (100%), 5'UTR:B0033m (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
   </si>
   <si>
     <t>promoter:J23107 (100%), RBS:B0034m (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
   </si>
   <si>
-    <t>promoter:J23103 (100%), 5'UTR:B0033m (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
-  </si>
-  <si>
-    <t>promoter:J23103 (100%), 5'UTR:BCD8 (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
+    <t>promoter:J23107 (100%), 5'UTR:BCD8 (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
   </si>
   <si>
     <t>promoter:J23116 (100%), RBS:B0034m (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
   </si>
   <si>
-    <t>promoter:J23103 (100%), 5'UTR:BCD12 (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
-  </si>
-  <si>
-    <t>promoter:J23106 (100%), 5'UTR:BCD8 (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
-  </si>
-  <si>
-    <t>promoter:J23107 (100%), 5'UTR:B0033m (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
-  </si>
-  <si>
     <t>promoter:J23116 (100%), 5'UTR:B0033m (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
   </si>
   <si>
-    <t>promoter:J23107 (100%), 5'UTR:BCD8 (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
-  </si>
-  <si>
     <t>promoter:J23106 (100%), 5'UTR:BCD12 (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
   </si>
   <si>
+    <t>promoter:R0010 (100%), RBS:B0034m (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
+  </si>
+  <si>
+    <t>promoter:R0010 (100%), 5'UTR:B0033m (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
+  </si>
+  <si>
     <t>promoter:J23116 (100%), 5'UTR:BCD8 (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
   </si>
   <si>
-    <t>promoter:R0010 (100%), RBS:B0034m (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
-  </si>
-  <si>
     <t>promoter:J23102 (100%), 5'UTR:B0032m (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
   </si>
   <si>
-    <t>promoter:R0010 (100%), 5'UTR:B0033m (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
+    <t>promoter:J23116 (100%), 5'UTR:BCD12 (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
+  </si>
+  <si>
+    <t>promoter:J23107 (100%), 5'UTR:BCD12 (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
   </si>
   <si>
     <t>promoter:J23100 (100%), 5'UTR:B0032m (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
   </si>
   <si>
-    <t>promoter:J23107 (100%), 5'UTR:BCD12 (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
+    <t>promoter:R0010 (100%), 5'UTR:BCD8 (100%), CDS:EcPanD (100%), misc_feature:B0015 (99%)</t>
   </si>
   <si>
     <t>promoter:J23102 (100%), RBS:B0034m (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
   </si>
   <si>
-    <t>promoter:J23116 (100%), 5'UTR:BCD12 (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
+    <t>promoter:J23102 (100%), 5'UTR:BCD8 (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
   </si>
   <si>
     <t>promoter:R0010 (100%), 5'UTR:BCD8 (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
   </si>
   <si>
-    <t>promoter:R0010 (100%), 5'UTR:BCD8 (100%), CDS:EcPanD (100%), misc_feature:B0015 (99%)</t>
+    <t>promoter:J23103 (100%), RBS:B0034m (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
+  </si>
+  <si>
+    <t>promoter:J23100 (100%), RBS:B0034m (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
   </si>
   <si>
     <t>promoter:R0010 (100%), 5'UTR:BCD12 (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
   </si>
   <si>
-    <t>promoter:J23103 (100%), RBS:B0034m (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
-  </si>
-  <si>
-    <t>promoter:J23102 (100%), 5'UTR:BCD8 (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
+    <t>promoter:J23102 (100%), 5'UTR:B0033m (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
   </si>
   <si>
     <t>promoter:J23106 (100%), 5'UTR:B0032m (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
   </si>
   <si>
-    <t>promoter:J23102 (100%), 5'UTR:B0033m (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
-  </si>
-  <si>
-    <t>promoter:J23100 (100%), RBS:B0034m (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
-  </si>
-  <si>
     <t>promoter:J23106 (100%), RBS:B0034m (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
   </si>
   <si>
@@ -589,22 +589,22 @@
     <t>0–565</t>
   </si>
   <si>
+    <t>0–629</t>
+  </si>
+  <si>
     <t>0–732</t>
   </si>
   <si>
-    <t>0–629</t>
-  </si>
-  <si>
     <t>0–566</t>
   </si>
   <si>
     <t>0–731</t>
   </si>
   <si>
+    <t>0–730</t>
+  </si>
+  <si>
     <t>0–567</t>
-  </si>
-  <si>
-    <t>0–730</t>
   </si>
   <si>
     <t>0–794</t>
@@ -982,7 +982,7 @@
     <col min="12" max="12" width="6.7109375" customWidth="1"/>
     <col min="13" max="13" width="80.7109375" customWidth="1"/>
     <col min="14" max="14" width="12.7109375" customWidth="1"/>
-    <col min="15" max="15" width="17.7109375" customWidth="1"/>
+    <col min="15" max="15" width="19.7109375" customWidth="1"/>
     <col min="16" max="16" width="9.7109375" customWidth="1"/>
     <col min="17" max="17" width="21.7109375" customWidth="1"/>
     <col min="18" max="18" width="12.7109375" customWidth="1"/>
@@ -1049,7 +1049,7 @@
         <v>18</v>
       </c>
       <c r="B2">
-        <v>1168</v>
+        <v>1186</v>
       </c>
       <c r="C2" t="s">
         <v>59</v>
@@ -1102,7 +1102,7 @@
         <v>19</v>
       </c>
       <c r="B3">
-        <v>1222</v>
+        <v>1235</v>
       </c>
       <c r="C3" t="s">
         <v>60</v>
@@ -1120,16 +1120,16 @@
         <v>1</v>
       </c>
       <c r="H3">
-        <v>744</v>
+        <v>641</v>
       </c>
       <c r="I3">
-        <v>723</v>
+        <v>620</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>732</v>
+        <v>629</v>
       </c>
       <c r="L3">
         <v>0</v>
@@ -1141,6 +1141,9 @@
         <v>190</v>
       </c>
       <c r="O3">
+        <v>100</v>
+      </c>
+      <c r="P3">
         <v>100</v>
       </c>
       <c r="Q3">
@@ -1155,7 +1158,7 @@
         <v>20</v>
       </c>
       <c r="B4">
-        <v>1235</v>
+        <v>1171</v>
       </c>
       <c r="C4" t="s">
         <v>61</v>
@@ -1191,9 +1194,12 @@
         <v>158</v>
       </c>
       <c r="N4" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="O4">
+        <v>100</v>
+      </c>
+      <c r="P4">
         <v>100</v>
       </c>
       <c r="Q4">
@@ -1208,7 +1214,7 @@
         <v>21</v>
       </c>
       <c r="B5">
-        <v>1175</v>
+        <v>1222</v>
       </c>
       <c r="C5" t="s">
         <v>62</v>
@@ -1226,16 +1232,16 @@
         <v>1</v>
       </c>
       <c r="H5">
-        <v>641</v>
+        <v>744</v>
       </c>
       <c r="I5">
-        <v>620</v>
+        <v>723</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>629</v>
+        <v>732</v>
       </c>
       <c r="L5">
         <v>0</v>
@@ -1261,7 +1267,7 @@
         <v>22</v>
       </c>
       <c r="B6">
-        <v>1186</v>
+        <v>1175</v>
       </c>
       <c r="C6" t="s">
         <v>63</v>
@@ -1279,16 +1285,16 @@
         <v>1</v>
       </c>
       <c r="H6">
-        <v>577</v>
+        <v>641</v>
       </c>
       <c r="I6">
-        <v>556</v>
+        <v>620</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>565</v>
+        <v>629</v>
       </c>
       <c r="L6">
         <v>0</v>
@@ -1297,9 +1303,12 @@
         <v>160</v>
       </c>
       <c r="N6" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="O6">
+        <v>100</v>
+      </c>
+      <c r="P6">
         <v>100</v>
       </c>
       <c r="Q6">
@@ -1314,7 +1323,7 @@
         <v>23</v>
       </c>
       <c r="B7">
-        <v>1196</v>
+        <v>1168</v>
       </c>
       <c r="C7" t="s">
         <v>64</v>
@@ -1332,16 +1341,16 @@
         <v>1</v>
       </c>
       <c r="H7">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="I7">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="L7">
         <v>0</v>
@@ -1350,7 +1359,7 @@
         <v>161</v>
       </c>
       <c r="N7" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="O7">
         <v>100</v>
@@ -1420,7 +1429,7 @@
         <v>25</v>
       </c>
       <c r="B9">
-        <v>1171</v>
+        <v>1175</v>
       </c>
       <c r="C9" t="s">
         <v>66</v>
@@ -1456,9 +1465,12 @@
         <v>163</v>
       </c>
       <c r="N9" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="O9">
+        <v>100</v>
+      </c>
+      <c r="P9">
         <v>100</v>
       </c>
       <c r="Q9">
@@ -1473,7 +1485,7 @@
         <v>26</v>
       </c>
       <c r="B10">
-        <v>1200</v>
+        <v>1210</v>
       </c>
       <c r="C10" t="s">
         <v>67</v>
@@ -1491,16 +1503,16 @@
         <v>1</v>
       </c>
       <c r="H10">
-        <v>578</v>
+        <v>641</v>
       </c>
       <c r="I10">
-        <v>557</v>
+        <v>620</v>
       </c>
       <c r="J10">
         <v>0</v>
       </c>
       <c r="K10">
-        <v>566</v>
+        <v>629</v>
       </c>
       <c r="L10">
         <v>0</v>
@@ -1509,9 +1521,12 @@
         <v>164</v>
       </c>
       <c r="N10" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="O10">
+        <v>100</v>
+      </c>
+      <c r="P10">
         <v>100</v>
       </c>
       <c r="Q10">
@@ -1526,7 +1541,7 @@
         <v>27</v>
       </c>
       <c r="B11">
-        <v>1210</v>
+        <v>1107</v>
       </c>
       <c r="C11" t="s">
         <v>68</v>
@@ -1544,16 +1559,16 @@
         <v>1</v>
       </c>
       <c r="H11">
-        <v>641</v>
+        <v>577</v>
       </c>
       <c r="I11">
-        <v>620</v>
+        <v>556</v>
       </c>
       <c r="J11">
         <v>0</v>
       </c>
       <c r="K11">
-        <v>629</v>
+        <v>565</v>
       </c>
       <c r="L11">
         <v>0</v>
@@ -1562,7 +1577,7 @@
         <v>165</v>
       </c>
       <c r="N11" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="O11">
         <v>100</v>
@@ -1579,7 +1594,7 @@
         <v>28</v>
       </c>
       <c r="B12">
-        <v>1175</v>
+        <v>1196</v>
       </c>
       <c r="C12" t="s">
         <v>69</v>
@@ -1597,16 +1612,16 @@
         <v>1</v>
       </c>
       <c r="H12">
-        <v>641</v>
+        <v>578</v>
       </c>
       <c r="I12">
-        <v>620</v>
+        <v>557</v>
       </c>
       <c r="J12">
         <v>0</v>
       </c>
       <c r="K12">
-        <v>629</v>
+        <v>566</v>
       </c>
       <c r="L12">
         <v>0</v>
@@ -1615,9 +1630,12 @@
         <v>166</v>
       </c>
       <c r="N12" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="O12">
+        <v>100</v>
+      </c>
+      <c r="P12">
         <v>100</v>
       </c>
       <c r="Q12">
@@ -1632,7 +1650,7 @@
         <v>29</v>
       </c>
       <c r="B13">
-        <v>1107</v>
+        <v>1171</v>
       </c>
       <c r="C13" t="s">
         <v>70</v>
@@ -1650,16 +1668,16 @@
         <v>1</v>
       </c>
       <c r="H13">
-        <v>577</v>
+        <v>641</v>
       </c>
       <c r="I13">
-        <v>556</v>
+        <v>620</v>
       </c>
       <c r="J13">
         <v>0</v>
       </c>
       <c r="K13">
-        <v>565</v>
+        <v>629</v>
       </c>
       <c r="L13">
         <v>0</v>
@@ -1668,9 +1686,12 @@
         <v>167</v>
       </c>
       <c r="N13" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="O13">
+        <v>100</v>
+      </c>
+      <c r="P13">
         <v>100</v>
       </c>
       <c r="Q13">
@@ -1685,16 +1706,16 @@
         <v>30</v>
       </c>
       <c r="B14">
-        <v>1177</v>
+        <v>1200</v>
       </c>
       <c r="C14" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="D14" t="s">
-        <v>92</v>
+        <v>103</v>
       </c>
       <c r="E14" t="s">
-        <v>124</v>
+        <v>135</v>
       </c>
       <c r="F14" t="s">
         <v>155</v>
@@ -1703,27 +1724,30 @@
         <v>1</v>
       </c>
       <c r="H14">
-        <v>744</v>
+        <v>578</v>
       </c>
       <c r="I14">
-        <v>723</v>
+        <v>557</v>
       </c>
       <c r="J14">
         <v>0</v>
       </c>
       <c r="K14">
-        <v>732</v>
+        <v>566</v>
       </c>
       <c r="L14">
         <v>0</v>
       </c>
       <c r="M14" t="s">
-        <v>157</v>
+        <v>168</v>
       </c>
       <c r="N14" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="O14">
+        <v>100</v>
+      </c>
+      <c r="P14">
         <v>100</v>
       </c>
       <c r="Q14">
@@ -1741,13 +1765,13 @@
         <v>1171</v>
       </c>
       <c r="C15" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D15" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E15" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F15" t="s">
         <v>155</v>
@@ -1771,7 +1795,7 @@
         <v>0</v>
       </c>
       <c r="M15" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="N15" t="s">
         <v>189</v>
@@ -1791,16 +1815,16 @@
         <v>32</v>
       </c>
       <c r="B16">
-        <v>1171</v>
+        <v>1110</v>
       </c>
       <c r="C16" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="D16" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="E16" t="s">
-        <v>136</v>
+        <v>128</v>
       </c>
       <c r="F16" t="s">
         <v>155</v>
@@ -1809,25 +1833,25 @@
         <v>1</v>
       </c>
       <c r="H16">
-        <v>641</v>
+        <v>577</v>
       </c>
       <c r="I16">
-        <v>620</v>
+        <v>556</v>
       </c>
       <c r="J16">
         <v>0</v>
       </c>
       <c r="K16">
-        <v>629</v>
+        <v>565</v>
       </c>
       <c r="L16">
         <v>0</v>
       </c>
       <c r="M16" t="s">
-        <v>169</v>
+        <v>161</v>
       </c>
       <c r="N16" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="O16">
         <v>100</v>
@@ -1844,16 +1868,16 @@
         <v>33</v>
       </c>
       <c r="B17">
-        <v>1237</v>
+        <v>1170</v>
       </c>
       <c r="C17" t="s">
-        <v>73</v>
+        <v>64</v>
       </c>
       <c r="D17" t="s">
-        <v>105</v>
+        <v>96</v>
       </c>
       <c r="E17" t="s">
-        <v>137</v>
+        <v>128</v>
       </c>
       <c r="F17" t="s">
         <v>155</v>
@@ -1862,25 +1886,25 @@
         <v>1</v>
       </c>
       <c r="H17">
-        <v>641</v>
+        <v>577</v>
       </c>
       <c r="I17">
-        <v>620</v>
+        <v>556</v>
       </c>
       <c r="J17">
         <v>0</v>
       </c>
       <c r="K17">
-        <v>629</v>
+        <v>565</v>
       </c>
       <c r="L17">
         <v>0</v>
       </c>
       <c r="M17" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="N17" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="O17">
         <v>100</v>
@@ -1897,16 +1921,16 @@
         <v>34</v>
       </c>
       <c r="B18">
-        <v>1110</v>
+        <v>1237</v>
       </c>
       <c r="C18" t="s">
-        <v>59</v>
+        <v>73</v>
       </c>
       <c r="D18" t="s">
-        <v>91</v>
+        <v>105</v>
       </c>
       <c r="E18" t="s">
-        <v>123</v>
+        <v>137</v>
       </c>
       <c r="F18" t="s">
         <v>155</v>
@@ -1915,27 +1939,30 @@
         <v>1</v>
       </c>
       <c r="H18">
-        <v>577</v>
+        <v>641</v>
       </c>
       <c r="I18">
-        <v>556</v>
+        <v>620</v>
       </c>
       <c r="J18">
         <v>0</v>
       </c>
       <c r="K18">
-        <v>565</v>
+        <v>629</v>
       </c>
       <c r="L18">
         <v>0</v>
       </c>
       <c r="M18" t="s">
-        <v>156</v>
+        <v>170</v>
       </c>
       <c r="N18" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="O18">
+        <v>100</v>
+      </c>
+      <c r="P18">
         <v>100</v>
       </c>
       <c r="Q18">
@@ -1950,16 +1977,16 @@
         <v>35</v>
       </c>
       <c r="B19">
-        <v>1174</v>
+        <v>1177</v>
       </c>
       <c r="C19" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="D19" t="s">
-        <v>106</v>
+        <v>94</v>
       </c>
       <c r="E19" t="s">
-        <v>138</v>
+        <v>126</v>
       </c>
       <c r="F19" t="s">
         <v>155</v>
@@ -1968,22 +1995,22 @@
         <v>1</v>
       </c>
       <c r="H19">
-        <v>641</v>
+        <v>744</v>
       </c>
       <c r="I19">
-        <v>620</v>
+        <v>723</v>
       </c>
       <c r="J19">
         <v>0</v>
       </c>
       <c r="K19">
-        <v>629</v>
+        <v>732</v>
       </c>
       <c r="L19">
         <v>0</v>
       </c>
       <c r="M19" t="s">
-        <v>171</v>
+        <v>159</v>
       </c>
       <c r="N19" t="s">
         <v>191</v>
@@ -2003,16 +2030,16 @@
         <v>36</v>
       </c>
       <c r="B20">
-        <v>1170</v>
+        <v>1184</v>
       </c>
       <c r="C20" t="s">
-        <v>59</v>
+        <v>74</v>
       </c>
       <c r="D20" t="s">
-        <v>91</v>
+        <v>106</v>
       </c>
       <c r="E20" t="s">
-        <v>123</v>
+        <v>138</v>
       </c>
       <c r="F20" t="s">
         <v>155</v>
@@ -2021,27 +2048,30 @@
         <v>1</v>
       </c>
       <c r="H20">
-        <v>577</v>
+        <v>743</v>
       </c>
       <c r="I20">
-        <v>556</v>
+        <v>722</v>
       </c>
       <c r="J20">
         <v>0</v>
       </c>
       <c r="K20">
-        <v>565</v>
+        <v>731</v>
       </c>
       <c r="L20">
         <v>0</v>
       </c>
       <c r="M20" t="s">
-        <v>156</v>
+        <v>171</v>
       </c>
       <c r="N20" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="O20">
+        <v>100</v>
+      </c>
+      <c r="P20">
         <v>100</v>
       </c>
       <c r="Q20">
@@ -2056,7 +2086,7 @@
         <v>37</v>
       </c>
       <c r="B21">
-        <v>1184</v>
+        <v>1240</v>
       </c>
       <c r="C21" t="s">
         <v>75</v>
@@ -2074,16 +2104,16 @@
         <v>1</v>
       </c>
       <c r="H21">
-        <v>743</v>
+        <v>742</v>
       </c>
       <c r="I21">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="J21">
         <v>0</v>
       </c>
       <c r="K21">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="L21">
         <v>0</v>
@@ -2092,7 +2122,7 @@
         <v>172</v>
       </c>
       <c r="N21" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="O21">
         <v>100</v>
@@ -2109,7 +2139,7 @@
         <v>38</v>
       </c>
       <c r="B22">
-        <v>1074</v>
+        <v>1174</v>
       </c>
       <c r="C22" t="s">
         <v>76</v>
@@ -2127,16 +2157,16 @@
         <v>1</v>
       </c>
       <c r="H22">
-        <v>579</v>
+        <v>641</v>
       </c>
       <c r="I22">
-        <v>558</v>
+        <v>620</v>
       </c>
       <c r="J22">
         <v>0</v>
       </c>
       <c r="K22">
-        <v>567</v>
+        <v>629</v>
       </c>
       <c r="L22">
         <v>0</v>
@@ -2145,9 +2175,12 @@
         <v>173</v>
       </c>
       <c r="N22" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="O22">
+        <v>100</v>
+      </c>
+      <c r="P22">
         <v>100</v>
       </c>
       <c r="Q22">
@@ -2162,7 +2195,7 @@
         <v>39</v>
       </c>
       <c r="B23">
-        <v>1240</v>
+        <v>1074</v>
       </c>
       <c r="C23" t="s">
         <v>77</v>
@@ -2180,16 +2213,16 @@
         <v>1</v>
       </c>
       <c r="H23">
-        <v>742</v>
+        <v>579</v>
       </c>
       <c r="I23">
-        <v>721</v>
+        <v>558</v>
       </c>
       <c r="J23">
         <v>0</v>
       </c>
       <c r="K23">
-        <v>730</v>
+        <v>567</v>
       </c>
       <c r="L23">
         <v>0</v>
@@ -2215,16 +2248,16 @@
         <v>40</v>
       </c>
       <c r="B24">
-        <v>1244</v>
+        <v>1173</v>
       </c>
       <c r="C24" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="D24" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="E24" t="s">
-        <v>135</v>
+        <v>142</v>
       </c>
       <c r="F24" t="s">
         <v>155</v>
@@ -2233,27 +2266,30 @@
         <v>1</v>
       </c>
       <c r="H24">
-        <v>577</v>
+        <v>641</v>
       </c>
       <c r="I24">
-        <v>556</v>
+        <v>620</v>
       </c>
       <c r="J24">
         <v>0</v>
       </c>
       <c r="K24">
-        <v>565</v>
+        <v>629</v>
       </c>
       <c r="L24">
         <v>0</v>
       </c>
       <c r="M24" t="s">
-        <v>168</v>
+        <v>175</v>
       </c>
       <c r="N24" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="O24">
+        <v>100</v>
+      </c>
+      <c r="P24">
         <v>100</v>
       </c>
       <c r="Q24">
@@ -2268,16 +2304,16 @@
         <v>41</v>
       </c>
       <c r="B25">
-        <v>1245</v>
+        <v>1235</v>
       </c>
       <c r="C25" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D25" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E25" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="F25" t="s">
         <v>155</v>
@@ -2286,27 +2322,30 @@
         <v>1</v>
       </c>
       <c r="H25">
-        <v>579</v>
+        <v>641</v>
       </c>
       <c r="I25">
-        <v>558</v>
+        <v>620</v>
       </c>
       <c r="J25">
         <v>0</v>
       </c>
       <c r="K25">
-        <v>567</v>
+        <v>629</v>
       </c>
       <c r="L25">
         <v>0</v>
       </c>
       <c r="M25" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="N25" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="O25">
+        <v>100</v>
+      </c>
+      <c r="P25">
         <v>100</v>
       </c>
       <c r="Q25">
@@ -2321,16 +2360,16 @@
         <v>42</v>
       </c>
       <c r="B26">
-        <v>1235</v>
+        <v>1244</v>
       </c>
       <c r="C26" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="D26" t="s">
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="E26" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="F26" t="s">
         <v>155</v>
@@ -2339,25 +2378,25 @@
         <v>1</v>
       </c>
       <c r="H26">
-        <v>641</v>
+        <v>577</v>
       </c>
       <c r="I26">
-        <v>620</v>
+        <v>556</v>
       </c>
       <c r="J26">
         <v>0</v>
       </c>
       <c r="K26">
-        <v>629</v>
+        <v>565</v>
       </c>
       <c r="L26">
         <v>0</v>
       </c>
       <c r="M26" t="s">
-        <v>176</v>
+        <v>169</v>
       </c>
       <c r="N26" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="O26">
         <v>100</v>
@@ -2374,16 +2413,16 @@
         <v>43</v>
       </c>
       <c r="B27">
-        <v>1189</v>
+        <v>1230</v>
       </c>
       <c r="C27" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="D27" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="E27" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="F27" t="s">
         <v>155</v>
@@ -2392,25 +2431,25 @@
         <v>1</v>
       </c>
       <c r="H27">
-        <v>578</v>
+        <v>742</v>
       </c>
       <c r="I27">
-        <v>557</v>
+        <v>721</v>
       </c>
       <c r="J27">
         <v>0</v>
       </c>
       <c r="K27">
-        <v>566</v>
+        <v>730</v>
       </c>
       <c r="L27">
         <v>0</v>
       </c>
       <c r="M27" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="N27" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="O27">
         <v>100</v>
@@ -2427,16 +2466,16 @@
         <v>44</v>
       </c>
       <c r="B28">
-        <v>1173</v>
+        <v>1245</v>
       </c>
       <c r="C28" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D28" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E28" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F28" t="s">
         <v>155</v>
@@ -2445,25 +2484,25 @@
         <v>1</v>
       </c>
       <c r="H28">
-        <v>641</v>
+        <v>579</v>
       </c>
       <c r="I28">
-        <v>620</v>
+        <v>558</v>
       </c>
       <c r="J28">
         <v>0</v>
       </c>
       <c r="K28">
-        <v>629</v>
+        <v>567</v>
       </c>
       <c r="L28">
         <v>0</v>
       </c>
       <c r="M28" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="N28" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="O28">
         <v>100</v>
@@ -2480,28 +2519,28 @@
         <v>45</v>
       </c>
       <c r="B29">
-        <v>1228</v>
+        <v>1163</v>
       </c>
       <c r="C29" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D29" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E29" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F29" t="s">
         <v>155</v>
       </c>
       <c r="G29">
-        <v>1</v>
+        <v>0.9987405541561712</v>
       </c>
       <c r="H29">
         <v>806</v>
       </c>
       <c r="I29">
-        <v>785</v>
+        <v>783</v>
       </c>
       <c r="J29">
         <v>0</v>
@@ -2510,15 +2549,18 @@
         <v>794</v>
       </c>
       <c r="L29">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M29" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="N29" t="s">
         <v>196</v>
       </c>
       <c r="O29">
+        <v>99.22480620155039</v>
+      </c>
+      <c r="P29">
         <v>100</v>
       </c>
       <c r="Q29">
@@ -2533,16 +2575,16 @@
         <v>46</v>
       </c>
       <c r="B30">
-        <v>1230</v>
+        <v>1189</v>
       </c>
       <c r="C30" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="D30" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="E30" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="F30" t="s">
         <v>155</v>
@@ -2551,27 +2593,30 @@
         <v>1</v>
       </c>
       <c r="H30">
-        <v>742</v>
+        <v>578</v>
       </c>
       <c r="I30">
-        <v>721</v>
+        <v>557</v>
       </c>
       <c r="J30">
         <v>0</v>
       </c>
       <c r="K30">
-        <v>730</v>
+        <v>566</v>
       </c>
       <c r="L30">
         <v>0</v>
       </c>
       <c r="M30" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="N30" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="O30">
+        <v>100</v>
+      </c>
+      <c r="P30">
         <v>100</v>
       </c>
       <c r="Q30">
@@ -2586,45 +2631,48 @@
         <v>47</v>
       </c>
       <c r="B31">
-        <v>1163</v>
+        <v>1171</v>
       </c>
       <c r="C31" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D31" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="E31" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F31" t="s">
         <v>155</v>
       </c>
       <c r="G31">
-        <v>0.9987405541561712</v>
+        <v>1</v>
       </c>
       <c r="H31">
-        <v>806</v>
+        <v>641</v>
       </c>
       <c r="I31">
-        <v>783</v>
+        <v>620</v>
       </c>
       <c r="J31">
         <v>0</v>
       </c>
       <c r="K31">
-        <v>794</v>
+        <v>629</v>
       </c>
       <c r="L31">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M31" t="s">
         <v>180</v>
       </c>
       <c r="N31" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="O31">
+        <v>100</v>
+      </c>
+      <c r="P31">
         <v>100</v>
       </c>
       <c r="Q31">
@@ -2642,25 +2690,25 @@
         <v>1228</v>
       </c>
       <c r="C32" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="D32" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="E32" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F32" t="s">
         <v>155</v>
       </c>
       <c r="G32">
-        <v>0.9987405541561712</v>
+        <v>1</v>
       </c>
       <c r="H32">
         <v>806</v>
       </c>
       <c r="I32">
-        <v>783</v>
+        <v>785</v>
       </c>
       <c r="J32">
         <v>0</v>
@@ -2669,7 +2717,7 @@
         <v>794</v>
       </c>
       <c r="L32">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M32" t="s">
         <v>181</v>
@@ -2678,6 +2726,9 @@
         <v>196</v>
       </c>
       <c r="O32">
+        <v>100</v>
+      </c>
+      <c r="P32">
         <v>100</v>
       </c>
       <c r="Q32">
@@ -2733,6 +2784,9 @@
       <c r="O33">
         <v>100</v>
       </c>
+      <c r="P33">
+        <v>100</v>
+      </c>
       <c r="Q33">
         <v>0</v>
       </c>
@@ -2745,16 +2799,16 @@
         <v>50</v>
       </c>
       <c r="B34">
-        <v>1240</v>
+        <v>1196</v>
       </c>
       <c r="C34" t="s">
-        <v>63</v>
+        <v>85</v>
       </c>
       <c r="D34" t="s">
-        <v>95</v>
+        <v>117</v>
       </c>
       <c r="E34" t="s">
-        <v>127</v>
+        <v>149</v>
       </c>
       <c r="F34" t="s">
         <v>155</v>
@@ -2763,27 +2817,30 @@
         <v>1</v>
       </c>
       <c r="H34">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="I34">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="J34">
         <v>0</v>
       </c>
       <c r="K34">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="L34">
         <v>0</v>
       </c>
       <c r="M34" t="s">
-        <v>160</v>
+        <v>183</v>
       </c>
       <c r="N34" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="O34">
+        <v>100</v>
+      </c>
+      <c r="P34">
         <v>100</v>
       </c>
       <c r="Q34">
@@ -2798,45 +2855,48 @@
         <v>51</v>
       </c>
       <c r="B35">
-        <v>1171</v>
+        <v>1228</v>
       </c>
       <c r="C35" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D35" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E35" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="F35" t="s">
         <v>155</v>
       </c>
       <c r="G35">
-        <v>1</v>
+        <v>0.9987405541561712</v>
       </c>
       <c r="H35">
-        <v>641</v>
+        <v>806</v>
       </c>
       <c r="I35">
-        <v>620</v>
+        <v>783</v>
       </c>
       <c r="J35">
         <v>0</v>
       </c>
       <c r="K35">
-        <v>629</v>
+        <v>794</v>
       </c>
       <c r="L35">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M35" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="N35" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
       <c r="O35">
+        <v>99.73753280839895</v>
+      </c>
+      <c r="P35">
         <v>100</v>
       </c>
       <c r="Q35">
@@ -2851,16 +2911,16 @@
         <v>52</v>
       </c>
       <c r="B36">
-        <v>1244</v>
+        <v>1242</v>
       </c>
       <c r="C36" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D36" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="E36" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="F36" t="s">
         <v>155</v>
@@ -2869,25 +2929,25 @@
         <v>1</v>
       </c>
       <c r="H36">
-        <v>579</v>
+        <v>577</v>
       </c>
       <c r="I36">
-        <v>558</v>
+        <v>556</v>
       </c>
       <c r="J36">
         <v>0</v>
       </c>
       <c r="K36">
-        <v>567</v>
+        <v>565</v>
       </c>
       <c r="L36">
         <v>0</v>
       </c>
       <c r="M36" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="N36" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="O36">
         <v>100</v>
@@ -2904,16 +2964,16 @@
         <v>53</v>
       </c>
       <c r="B37">
-        <v>1242</v>
+        <v>1244</v>
       </c>
       <c r="C37" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D37" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="E37" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F37" t="s">
         <v>155</v>
@@ -2922,25 +2982,25 @@
         <v>1</v>
       </c>
       <c r="H37">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="I37">
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="J37">
         <v>0</v>
       </c>
       <c r="K37">
-        <v>565</v>
+        <v>567</v>
       </c>
       <c r="L37">
         <v>0</v>
       </c>
       <c r="M37" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="N37" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
       <c r="O37">
         <v>100</v>
@@ -2957,16 +3017,16 @@
         <v>54</v>
       </c>
       <c r="B38">
-        <v>1201</v>
+        <v>1193</v>
       </c>
       <c r="C38" t="s">
-        <v>65</v>
+        <v>89</v>
       </c>
       <c r="D38" t="s">
-        <v>97</v>
+        <v>121</v>
       </c>
       <c r="E38" t="s">
-        <v>129</v>
+        <v>153</v>
       </c>
       <c r="F38" t="s">
         <v>155</v>
@@ -2975,27 +3035,30 @@
         <v>1</v>
       </c>
       <c r="H38">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="I38">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="J38">
         <v>0</v>
       </c>
       <c r="K38">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="L38">
         <v>0</v>
       </c>
       <c r="M38" t="s">
-        <v>162</v>
+        <v>187</v>
       </c>
       <c r="N38" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="O38">
+        <v>100</v>
+      </c>
+      <c r="P38">
         <v>100</v>
       </c>
       <c r="Q38">
@@ -3010,16 +3073,16 @@
         <v>55</v>
       </c>
       <c r="B39">
-        <v>1196</v>
+        <v>1240</v>
       </c>
       <c r="C39" t="s">
-        <v>88</v>
+        <v>59</v>
       </c>
       <c r="D39" t="s">
-        <v>120</v>
+        <v>91</v>
       </c>
       <c r="E39" t="s">
-        <v>152</v>
+        <v>123</v>
       </c>
       <c r="F39" t="s">
         <v>155</v>
@@ -3028,25 +3091,25 @@
         <v>1</v>
       </c>
       <c r="H39">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="I39">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="J39">
         <v>0</v>
       </c>
       <c r="K39">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="L39">
         <v>0</v>
       </c>
       <c r="M39" t="s">
-        <v>186</v>
+        <v>156</v>
       </c>
       <c r="N39" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="O39">
         <v>100</v>
@@ -3063,16 +3126,16 @@
         <v>56</v>
       </c>
       <c r="B40">
-        <v>1191</v>
+        <v>1203</v>
       </c>
       <c r="C40" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="D40" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="E40" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="F40" t="s">
         <v>155</v>
@@ -3081,25 +3144,25 @@
         <v>1</v>
       </c>
       <c r="H40">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="I40">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="J40">
         <v>0</v>
       </c>
       <c r="K40">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="L40">
         <v>0</v>
       </c>
       <c r="M40" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="N40" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="O40">
         <v>100</v>
@@ -3116,16 +3179,16 @@
         <v>57</v>
       </c>
       <c r="B41">
-        <v>1193</v>
+        <v>1201</v>
       </c>
       <c r="C41" t="s">
-        <v>89</v>
+        <v>65</v>
       </c>
       <c r="D41" t="s">
-        <v>121</v>
+        <v>97</v>
       </c>
       <c r="E41" t="s">
-        <v>153</v>
+        <v>129</v>
       </c>
       <c r="F41" t="s">
         <v>155</v>
@@ -3134,25 +3197,25 @@
         <v>1</v>
       </c>
       <c r="H41">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="I41">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="J41">
         <v>0</v>
       </c>
       <c r="K41">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="L41">
         <v>0</v>
       </c>
       <c r="M41" t="s">
-        <v>187</v>
+        <v>162</v>
       </c>
       <c r="N41" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="O41">
         <v>100</v>
@@ -3169,16 +3232,16 @@
         <v>58</v>
       </c>
       <c r="B42">
-        <v>1203</v>
+        <v>1191</v>
       </c>
       <c r="C42" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="D42" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="E42" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="F42" t="s">
         <v>155</v>
@@ -3187,27 +3250,30 @@
         <v>1</v>
       </c>
       <c r="H42">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="I42">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="J42">
         <v>0</v>
       </c>
       <c r="K42">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="L42">
         <v>0</v>
       </c>
       <c r="M42" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
       <c r="N42" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="O42">
+        <v>100</v>
+      </c>
+      <c r="P42">
         <v>100</v>
       </c>
       <c r="Q42">

</xml_diff>

<commit_message>
Add multi-TU sequencing verification example; refresh Golden Gate/Sequencing examples
- New example "03 Sequencing/05 Multi-TU alignment": per-TU-window alignment
  workflow for plasmids with multiple transcriptional units, validated against
  real long-read (Nanopore) assembly data for 4 constructs (R28/R9/R10 pathway
  plasmids + pJYS3_IS61_AE_Amp Cas12a plasmid). Includes classic plot_alignment/
  view_alignment_html visualizations.
- Add "02 insilico Plasmid Construction/06 Golden Gate diverse file types"
  example (mixed .dna/.gb inputs, automated Golden Gate assembly test).
- Refresh regenerated outputs in "03 Sequencing/02 From folder" example.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/03 Sequencing/02 From folder/alignment_results.xlsx
+++ b/examples/03 Sequencing/02 From folder/alignment_results.xlsx
@@ -76,165 +76,165 @@
     <t>EF73802034_EF73802034</t>
   </si>
   <si>
+    <t>EF73802037_EF73802037</t>
+  </si>
+  <si>
+    <t>EF73802046_EF73802046</t>
+  </si>
+  <si>
+    <t>EF73802036_EF73802036</t>
+  </si>
+  <si>
+    <t>EF73802035_EF73802035</t>
+  </si>
+  <si>
+    <t>EF73802047_EF73802047</t>
+  </si>
+  <si>
+    <t>EF73802038_EF73802038</t>
+  </si>
+  <si>
+    <t>EF73802049_EF73802049</t>
+  </si>
+  <si>
     <t>EF73802045_EF73802045</t>
   </si>
   <si>
-    <t>EF73802035_EF73802035</t>
-  </si>
-  <si>
-    <t>EF73802038_EF73802038</t>
-  </si>
-  <si>
-    <t>EF73802047_EF73802047</t>
-  </si>
-  <si>
-    <t>EF73802036_EF73802036</t>
-  </si>
-  <si>
-    <t>EF73802046_EF73802046</t>
+    <t>EF73802057_EF73802057</t>
   </si>
   <si>
     <t>EF73802033_EF73802033</t>
   </si>
   <si>
-    <t>EF73802057_EF73802057</t>
+    <t>EF73802058_EF73802058</t>
   </si>
   <si>
     <t>EF73802048_EF73802048</t>
   </si>
   <si>
-    <t>EF73802037_EF73802037</t>
-  </si>
-  <si>
     <t>EF73802059_EF73802059</t>
   </si>
   <si>
-    <t>EF73802049_EF73802049</t>
-  </si>
-  <si>
     <t>EF73802060_EF73802060</t>
   </si>
   <si>
-    <t>EF73802058_EF73802058</t>
+    <t>EF73802069_EF73802069</t>
+  </si>
+  <si>
+    <t>EF73802050_EF73802050</t>
+  </si>
+  <si>
+    <t>EF73802061_EF73802061</t>
   </si>
   <si>
     <t>EF73802070_EF73802070</t>
   </si>
   <si>
-    <t>EF73802069_EF73802069</t>
-  </si>
-  <si>
-    <t>EF73802050_EF73802050</t>
-  </si>
-  <si>
-    <t>EF73802061_EF73802061</t>
+    <t>EF73802071_EF73802071</t>
+  </si>
+  <si>
+    <t>EF73802081_EF73802081</t>
+  </si>
+  <si>
+    <t>EF73802083_EF73802083</t>
+  </si>
+  <si>
+    <t>EF73802084_EF73802084</t>
   </si>
   <si>
     <t>EF73802072_EF73802072</t>
   </si>
   <si>
-    <t>EF73802071_EF73802071</t>
+    <t>EF73802082_EF73802082</t>
   </si>
   <si>
     <t>EF73802073_EF73802073</t>
   </si>
   <si>
+    <t>EF73802105_EF73802105</t>
+  </si>
+  <si>
+    <t>EF73802106_EF73802106</t>
+  </si>
+  <si>
+    <t>EF73802085_EF73802085</t>
+  </si>
+  <si>
+    <t>EF73802096_EF73802096</t>
+  </si>
+  <si>
     <t>EF73802093_EF73802093</t>
   </si>
   <si>
-    <t>EF73802081_EF73802081</t>
-  </si>
-  <si>
-    <t>EF73802082_EF73802082</t>
-  </si>
-  <si>
     <t>EF73802094_EF73802094</t>
   </si>
   <si>
-    <t>EF73802085_EF73802085</t>
-  </si>
-  <si>
-    <t>EF73802083_EF73802083</t>
-  </si>
-  <si>
-    <t>EF73802084_EF73802084</t>
-  </si>
-  <si>
-    <t>EF73802106_EF73802106</t>
+    <t>EF73802130_EF73802130</t>
   </si>
   <si>
     <t>EF73802095_EF73802095</t>
   </si>
   <si>
+    <t>EF73802107_EF73802107</t>
+  </si>
+  <si>
+    <t>EF73802132_EF73802132</t>
+  </si>
+  <si>
+    <t>EF73802133_EF73802133</t>
+  </si>
+  <si>
     <t>EF73802108_EF73802108</t>
   </si>
   <si>
-    <t>EF73802096_EF73802096</t>
-  </si>
-  <si>
-    <t>EF73802105_EF73802105</t>
+    <t>EF73802131_EF73802131</t>
+  </si>
+  <si>
+    <t>EF73802109_EF73802109</t>
   </si>
   <si>
     <t>EF73802129_EF73802129</t>
   </si>
   <si>
-    <t>EF73802109_EF73802109</t>
-  </si>
-  <si>
-    <t>EF73802130_EF73802130</t>
-  </si>
-  <si>
-    <t>EF73802107_EF73802107</t>
-  </si>
-  <si>
-    <t>EF73802133_EF73802133</t>
-  </si>
-  <si>
-    <t>EF73802131_EF73802131</t>
-  </si>
-  <si>
-    <t>EF73802132_EF73802132</t>
-  </si>
-  <si>
     <t>J23100_AB_B0033m_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
   </si>
   <si>
+    <t>J23107_AB_B0034m_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
+  </si>
+  <si>
+    <t>J23103_AB_B0033m_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
+  </si>
+  <si>
+    <t>J23106_AB_B0033m_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
+  </si>
+  <si>
+    <t>J23103_AB_BCD8_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
+  </si>
+  <si>
+    <t>J23106_AB_BCD8_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
+  </si>
+  <si>
+    <t>R0010_AB_B0032m_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
+  </si>
+  <si>
+    <t>J23116_AB_B0034m_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
+  </si>
+  <si>
     <t>J23100_AB_BCD12_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
   </si>
   <si>
-    <t>J23103_AB_BCD8_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
-  </si>
-  <si>
-    <t>R0010_AB_B0032m_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
-  </si>
-  <si>
-    <t>J23106_AB_BCD8_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
-  </si>
-  <si>
-    <t>J23106_AB_B0033m_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
-  </si>
-  <si>
-    <t>J23103_AB_B0033m_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
+    <t>J23103_AB_BCD12_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
   </si>
   <si>
     <t>J23102_AB_BCD12_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
   </si>
   <si>
-    <t>J23103_AB_BCD12_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
-  </si>
-  <si>
     <t>J23107_AB_B0033m_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
   </si>
   <si>
-    <t>J23107_AB_B0034m_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
-  </si>
-  <si>
     <t>J23107_AB_BCD8_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
   </si>
   <si>
-    <t>J23116_AB_B0034m_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
-  </si>
-  <si>
     <t>J23116_AB_B0033m_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
   </si>
   <si>
@@ -244,93 +244,93 @@
     <t>R0010_AB_B0034m_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
   </si>
   <si>
+    <t>J23116_AB_BCD8_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
+  </si>
+  <si>
+    <t>J23107_AB_BCD12_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
+  </si>
+  <si>
+    <t>R0010_AB_BCD8_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
+  </si>
+  <si>
+    <t>J23102_AB_B0034m_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
+  </si>
+  <si>
     <t>R0010_AB_B0033m_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
   </si>
   <si>
-    <t>J23116_AB_BCD8_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
-  </si>
-  <si>
     <t>J23102_AB_B0032m_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
   </si>
   <si>
+    <t>R0010_AB_BCD12_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
+  </si>
+  <si>
+    <t>J23102_AB_BCD8_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
+  </si>
+  <si>
+    <t>J23100_AB_B0032m_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
+  </si>
+  <si>
+    <t>J23100_AB_B0034m_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
+  </si>
+  <si>
     <t>J23116_AB_BCD12_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
   </si>
   <si>
-    <t>J23107_AB_BCD12_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
-  </si>
-  <si>
-    <t>J23100_AB_B0032m_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
-  </si>
-  <si>
-    <t>R0010_AB_BCD8_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
-  </si>
-  <si>
-    <t>J23102_AB_B0034m_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
-  </si>
-  <si>
-    <t>J23102_AB_BCD8_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
+    <t>J23106_AB_B0034m_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
   </si>
   <si>
     <t>J23103_AB_B0034m_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
   </si>
   <si>
-    <t>J23100_AB_B0034m_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
-  </si>
-  <si>
-    <t>R0010_AB_BCD12_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
+    <t>J23107_AB_B0032m_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
+  </si>
+  <si>
+    <t>J23106_AB_B0032m_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
   </si>
   <si>
     <t>J23102_AB_B0033m_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
   </si>
   <si>
-    <t>J23106_AB_B0032m_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
-  </si>
-  <si>
-    <t>J23106_AB_B0034m_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
-  </si>
-  <si>
-    <t>J23107_AB_B0032m_BC_DVA_ecPanD_B0015_DF_DVK_AF.gb</t>
-  </si>
-  <si>
     <t>J23100_AB_B0033m_BC_</t>
   </si>
   <si>
+    <t>J23107_AB_B0034m_BC_</t>
+  </si>
+  <si>
+    <t>J23103_AB_B0033m_BC_</t>
+  </si>
+  <si>
+    <t>J23106_AB_B0033m_BC_</t>
+  </si>
+  <si>
+    <t>J23103_AB_BCD8_BC_DV</t>
+  </si>
+  <si>
+    <t>J23106_AB_BCD8_BC_DV</t>
+  </si>
+  <si>
+    <t>R0010_AB_B0032m_BC_D</t>
+  </si>
+  <si>
+    <t>J23116_AB_B0034m_BC_</t>
+  </si>
+  <si>
     <t>J23100_AB_BCD12_BC_D</t>
   </si>
   <si>
-    <t>J23103_AB_BCD8_BC_DV</t>
-  </si>
-  <si>
-    <t>R0010_AB_B0032m_BC_D</t>
-  </si>
-  <si>
-    <t>J23106_AB_BCD8_BC_DV</t>
-  </si>
-  <si>
-    <t>J23106_AB_B0033m_BC_</t>
-  </si>
-  <si>
-    <t>J23103_AB_B0033m_BC_</t>
+    <t>J23103_AB_BCD12_BC_D</t>
   </si>
   <si>
     <t>J23102_AB_BCD12_BC_D</t>
   </si>
   <si>
-    <t>J23103_AB_BCD12_BC_D</t>
-  </si>
-  <si>
     <t>J23107_AB_B0033m_BC_</t>
   </si>
   <si>
-    <t>J23107_AB_B0034m_BC_</t>
-  </si>
-  <si>
     <t>J23107_AB_BCD8_BC_DV</t>
   </si>
   <si>
-    <t>J23116_AB_B0034m_BC_</t>
-  </si>
-  <si>
     <t>J23116_AB_B0033m_BC_</t>
   </si>
   <si>
@@ -340,93 +340,93 @@
     <t>R0010_AB_B0034m_BC_D</t>
   </si>
   <si>
+    <t>J23116_AB_BCD8_BC_DV</t>
+  </si>
+  <si>
+    <t>J23107_AB_BCD12_BC_D</t>
+  </si>
+  <si>
+    <t>R0010_AB_BCD8_BC_DVA</t>
+  </si>
+  <si>
+    <t>J23102_AB_B0034m_BC_</t>
+  </si>
+  <si>
     <t>R0010_AB_B0033m_BC_D</t>
   </si>
   <si>
-    <t>J23116_AB_BCD8_BC_DV</t>
-  </si>
-  <si>
     <t>J23102_AB_B0032m_BC_</t>
   </si>
   <si>
+    <t>R0010_AB_BCD12_BC_DV</t>
+  </si>
+  <si>
+    <t>J23102_AB_BCD8_BC_DV</t>
+  </si>
+  <si>
+    <t>J23100_AB_B0032m_BC_</t>
+  </si>
+  <si>
+    <t>J23100_AB_B0034m_BC_</t>
+  </si>
+  <si>
     <t>J23116_AB_BCD12_BC_D</t>
   </si>
   <si>
-    <t>J23107_AB_BCD12_BC_D</t>
-  </si>
-  <si>
-    <t>J23100_AB_B0032m_BC_</t>
-  </si>
-  <si>
-    <t>R0010_AB_BCD8_BC_DVA</t>
-  </si>
-  <si>
-    <t>J23102_AB_B0034m_BC_</t>
-  </si>
-  <si>
-    <t>J23102_AB_BCD8_BC_DV</t>
+    <t>J23106_AB_B0034m_BC_</t>
   </si>
   <si>
     <t>J23103_AB_B0034m_BC_</t>
   </si>
   <si>
-    <t>J23100_AB_B0034m_BC_</t>
-  </si>
-  <si>
-    <t>R0010_AB_BCD12_BC_DV</t>
+    <t>J23107_AB_B0032m_BC_</t>
+  </si>
+  <si>
+    <t>J23106_AB_B0032m_BC_</t>
   </si>
   <si>
     <t>J23102_AB_B0033m_BC_</t>
   </si>
   <si>
-    <t>J23106_AB_B0032m_BC_</t>
-  </si>
-  <si>
-    <t>J23106_AB_B0034m_BC_</t>
-  </si>
-  <si>
-    <t>J23107_AB_B0032m_BC_</t>
-  </si>
-  <si>
     <t>J23100_B0033m_ecPanD_B0015</t>
   </si>
   <si>
+    <t>J23107_B0034m_ecPanD_B0015</t>
+  </si>
+  <si>
+    <t>J23103_B0033m_ecPanD_B0015</t>
+  </si>
+  <si>
+    <t>J23106_B0033m_ecPanD_B0015</t>
+  </si>
+  <si>
+    <t>J23103_BCD8_ecPanD_B0015</t>
+  </si>
+  <si>
+    <t>J23106_BCD8_ecPanD_B0015</t>
+  </si>
+  <si>
+    <t>B0032m_ecPanD_B0015</t>
+  </si>
+  <si>
+    <t>J23116_B0034m_ecPanD_B0015</t>
+  </si>
+  <si>
     <t>J23100_BCD12_ecPanD_B0015</t>
   </si>
   <si>
-    <t>J23103_BCD8_ecPanD_B0015</t>
-  </si>
-  <si>
-    <t>B0032m_ecPanD_B0015</t>
-  </si>
-  <si>
-    <t>J23106_BCD8_ecPanD_B0015</t>
-  </si>
-  <si>
-    <t>J23106_B0033m_ecPanD_B0015</t>
-  </si>
-  <si>
-    <t>J23103_B0033m_ecPanD_B0015</t>
+    <t>J23103_BCD12_ecPanD_B0015</t>
   </si>
   <si>
     <t>J23102_BCD12_ecPanD_B0015</t>
   </si>
   <si>
-    <t>J23103_BCD12_ecPanD_B0015</t>
-  </si>
-  <si>
     <t>J23107_B0033m_ecPanD_B0015</t>
   </si>
   <si>
-    <t>J23107_B0034m_ecPanD_B0015</t>
-  </si>
-  <si>
     <t>J23107_BCD8_ecPanD_B0015</t>
   </si>
   <si>
-    <t>J23116_B0034m_ecPanD_B0015</t>
-  </si>
-  <si>
     <t>J23116_B0033m_ecPanD_B0015</t>
   </si>
   <si>
@@ -436,96 +436,96 @@
     <t>B0034m_ecPanD_B0015</t>
   </si>
   <si>
+    <t>J23116_BCD8_ecPanD_B0015</t>
+  </si>
+  <si>
+    <t>J23107_BCD12_ecPanD_B0015</t>
+  </si>
+  <si>
+    <t>BCD8_ecPanD_B0015</t>
+  </si>
+  <si>
+    <t>J23102_B0034m_ecPanD_B0015</t>
+  </si>
+  <si>
     <t>B0033m_ecPanD_B0015</t>
   </si>
   <si>
-    <t>J23116_BCD8_ecPanD_B0015</t>
-  </si>
-  <si>
     <t>J23102_B0032m_ecPanD_B0015</t>
   </si>
   <si>
+    <t>BCD12_ecPanD_B0015</t>
+  </si>
+  <si>
+    <t>J23102_BCD8_ecPanD_B0015</t>
+  </si>
+  <si>
+    <t>J23100_B0032m_ecPanD_B0015</t>
+  </si>
+  <si>
+    <t>J23100_B0034m_ecPanD_B0015</t>
+  </si>
+  <si>
     <t>J23116_BCD12_ecPanD_B0015</t>
   </si>
   <si>
-    <t>J23107_BCD12_ecPanD_B0015</t>
-  </si>
-  <si>
-    <t>J23100_B0032m_ecPanD_B0015</t>
-  </si>
-  <si>
-    <t>BCD8_ecPanD_B0015</t>
-  </si>
-  <si>
-    <t>J23102_B0034m_ecPanD_B0015</t>
-  </si>
-  <si>
-    <t>J23102_BCD8_ecPanD_B0015</t>
+    <t>J23106_B0034m_ecPanD_B0015</t>
   </si>
   <si>
     <t>J23103_B0034m_ecPanD_B0015</t>
   </si>
   <si>
-    <t>J23100_B0034m_ecPanD_B0015</t>
-  </si>
-  <si>
-    <t>BCD12_ecPanD_B0015</t>
+    <t>J23107_B0032m_ecPanD_B0015</t>
+  </si>
+  <si>
+    <t>J23106_B0032m_ecPanD_B0015</t>
   </si>
   <si>
     <t>J23102_B0033m_ecPanD_B0015</t>
   </si>
   <si>
-    <t>J23106_B0032m_ecPanD_B0015</t>
-  </si>
-  <si>
-    <t>J23106_B0034m_ecPanD_B0015</t>
-  </si>
-  <si>
-    <t>J23107_B0032m_ecPanD_B0015</t>
-  </si>
-  <si>
     <t>F</t>
   </si>
   <si>
     <t>promoter:J23100 (100%), 5'UTR:B0033m (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
   </si>
   <si>
+    <t>promoter:J23107 (100%), RBS:B0034m (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
+  </si>
+  <si>
+    <t>promoter:J23103 (100%), 5'UTR:B0033m (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
+  </si>
+  <si>
+    <t>promoter:J23106 (100%), 5'UTR:B0033m (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
+  </si>
+  <si>
+    <t>promoter:J23103 (100%), 5'UTR:BCD8 (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
+  </si>
+  <si>
+    <t>promoter:J23106 (100%), 5'UTR:BCD8 (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
+  </si>
+  <si>
+    <t>promoter:R0010 (100%), 5'UTR:B0032m (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
+  </si>
+  <si>
+    <t>promoter:J23116 (100%), RBS:B0034m (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
+  </si>
+  <si>
     <t>promoter:J23100 (100%), 5'UTR:BCD12 (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
   </si>
   <si>
-    <t>promoter:J23103 (100%), 5'UTR:BCD8 (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
-  </si>
-  <si>
-    <t>promoter:R0010 (100%), 5'UTR:B0032m (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
-  </si>
-  <si>
-    <t>promoter:J23106 (100%), 5'UTR:BCD8 (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
-  </si>
-  <si>
-    <t>promoter:J23106 (100%), 5'UTR:B0033m (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
-  </si>
-  <si>
-    <t>promoter:J23103 (100%), 5'UTR:B0033m (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
+    <t>promoter:J23103 (100%), 5'UTR:BCD12 (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
   </si>
   <si>
     <t>promoter:J23102 (100%), 5'UTR:BCD12 (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
   </si>
   <si>
-    <t>promoter:J23103 (100%), 5'UTR:BCD12 (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
-  </si>
-  <si>
     <t>promoter:J23107 (100%), 5'UTR:B0033m (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
   </si>
   <si>
-    <t>promoter:J23107 (100%), RBS:B0034m (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
-  </si>
-  <si>
     <t>promoter:J23107 (100%), 5'UTR:BCD8 (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
   </si>
   <si>
-    <t>promoter:J23116 (100%), RBS:B0034m (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
-  </si>
-  <si>
     <t>promoter:J23116 (100%), 5'UTR:B0033m (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
   </si>
   <si>
@@ -535,31 +535,40 @@
     <t>promoter:R0010 (100%), RBS:B0034m (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
   </si>
   <si>
+    <t>promoter:J23116 (100%), 5'UTR:BCD8 (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
+  </si>
+  <si>
+    <t>promoter:J23107 (100%), 5'UTR:BCD12 (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
+  </si>
+  <si>
+    <t>promoter:R0010 (100%), 5'UTR:BCD8 (100%), CDS:EcPanD (100%), misc_feature:B0015 (99%)</t>
+  </si>
+  <si>
+    <t>promoter:J23102 (100%), RBS:B0034m (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
+  </si>
+  <si>
     <t>promoter:R0010 (100%), 5'UTR:B0033m (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
   </si>
   <si>
-    <t>promoter:J23116 (100%), 5'UTR:BCD8 (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
-  </si>
-  <si>
     <t>promoter:J23102 (100%), 5'UTR:B0032m (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
   </si>
   <si>
+    <t>promoter:R0010 (100%), 5'UTR:BCD12 (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
+  </si>
+  <si>
+    <t>promoter:J23102 (100%), 5'UTR:BCD8 (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
+  </si>
+  <si>
+    <t>promoter:J23100 (100%), 5'UTR:B0032m (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
+  </si>
+  <si>
+    <t>promoter:J23100 (100%), RBS:B0034m (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
+  </si>
+  <si>
     <t>promoter:J23116 (100%), 5'UTR:BCD12 (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
   </si>
   <si>
-    <t>promoter:J23107 (100%), 5'UTR:BCD12 (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
-  </si>
-  <si>
-    <t>promoter:J23100 (100%), 5'UTR:B0032m (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
-  </si>
-  <si>
-    <t>promoter:R0010 (100%), 5'UTR:BCD8 (100%), CDS:EcPanD (100%), misc_feature:B0015 (99%)</t>
-  </si>
-  <si>
-    <t>promoter:J23102 (100%), RBS:B0034m (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
-  </si>
-  <si>
-    <t>promoter:J23102 (100%), 5'UTR:BCD8 (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
+    <t>promoter:J23106 (100%), RBS:B0034m (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
   </si>
   <si>
     <t>promoter:R0010 (100%), 5'UTR:BCD8 (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
@@ -568,46 +577,37 @@
     <t>promoter:J23103 (100%), RBS:B0034m (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
   </si>
   <si>
-    <t>promoter:J23100 (100%), RBS:B0034m (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
-  </si>
-  <si>
-    <t>promoter:R0010 (100%), 5'UTR:BCD12 (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
+    <t>promoter:J23107 (100%), 5'UTR:B0032m (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
+  </si>
+  <si>
+    <t>promoter:J23106 (100%), 5'UTR:B0032m (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
   </si>
   <si>
     <t>promoter:J23102 (100%), 5'UTR:B0033m (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
   </si>
   <si>
-    <t>promoter:J23106 (100%), 5'UTR:B0032m (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
-  </si>
-  <si>
-    <t>promoter:J23106 (100%), RBS:B0034m (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
-  </si>
-  <si>
-    <t>promoter:J23107 (100%), 5'UTR:B0032m (100%), CDS:EcPanD (100%), misc_feature:B0015 (100%)</t>
-  </si>
-  <si>
     <t>0–565</t>
   </si>
   <si>
+    <t>0–566</t>
+  </si>
+  <si>
     <t>0–629</t>
   </si>
   <si>
     <t>0–732</t>
   </si>
   <si>
-    <t>0–566</t>
-  </si>
-  <si>
     <t>0–731</t>
   </si>
   <si>
+    <t>0–794</t>
+  </si>
+  <si>
     <t>0–730</t>
   </si>
   <si>
     <t>0–567</t>
-  </si>
-  <si>
-    <t>0–794</t>
   </si>
 </sst>
 </file>
@@ -1102,7 +1102,7 @@
         <v>19</v>
       </c>
       <c r="B3">
-        <v>1235</v>
+        <v>1196</v>
       </c>
       <c r="C3" t="s">
         <v>60</v>
@@ -1120,16 +1120,16 @@
         <v>1</v>
       </c>
       <c r="H3">
-        <v>641</v>
+        <v>578</v>
       </c>
       <c r="I3">
-        <v>620</v>
+        <v>557</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>629</v>
+        <v>566</v>
       </c>
       <c r="L3">
         <v>0</v>
@@ -1158,7 +1158,7 @@
         <v>20</v>
       </c>
       <c r="B4">
-        <v>1171</v>
+        <v>1174</v>
       </c>
       <c r="C4" t="s">
         <v>61</v>
@@ -1176,16 +1176,16 @@
         <v>1</v>
       </c>
       <c r="H4">
-        <v>641</v>
+        <v>577</v>
       </c>
       <c r="I4">
-        <v>620</v>
+        <v>556</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>629</v>
+        <v>565</v>
       </c>
       <c r="L4">
         <v>0</v>
@@ -1194,12 +1194,9 @@
         <v>158</v>
       </c>
       <c r="N4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="O4">
-        <v>100</v>
-      </c>
-      <c r="P4">
         <v>100</v>
       </c>
       <c r="Q4">
@@ -1214,7 +1211,7 @@
         <v>21</v>
       </c>
       <c r="B5">
-        <v>1222</v>
+        <v>1168</v>
       </c>
       <c r="C5" t="s">
         <v>62</v>
@@ -1232,16 +1229,16 @@
         <v>1</v>
       </c>
       <c r="H5">
-        <v>744</v>
+        <v>577</v>
       </c>
       <c r="I5">
-        <v>723</v>
+        <v>556</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>732</v>
+        <v>565</v>
       </c>
       <c r="L5">
         <v>0</v>
@@ -1250,7 +1247,7 @@
         <v>159</v>
       </c>
       <c r="N5" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="O5">
         <v>100</v>
@@ -1267,7 +1264,7 @@
         <v>22</v>
       </c>
       <c r="B6">
-        <v>1175</v>
+        <v>1171</v>
       </c>
       <c r="C6" t="s">
         <v>63</v>
@@ -1303,7 +1300,7 @@
         <v>160</v>
       </c>
       <c r="N6" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="O6">
         <v>100</v>
@@ -1323,7 +1320,7 @@
         <v>23</v>
       </c>
       <c r="B7">
-        <v>1168</v>
+        <v>1175</v>
       </c>
       <c r="C7" t="s">
         <v>64</v>
@@ -1341,16 +1338,16 @@
         <v>1</v>
       </c>
       <c r="H7">
-        <v>577</v>
+        <v>641</v>
       </c>
       <c r="I7">
-        <v>556</v>
+        <v>620</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>565</v>
+        <v>629</v>
       </c>
       <c r="L7">
         <v>0</v>
@@ -1359,9 +1356,12 @@
         <v>161</v>
       </c>
       <c r="N7" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="O7">
+        <v>100</v>
+      </c>
+      <c r="P7">
         <v>100</v>
       </c>
       <c r="Q7">
@@ -1376,7 +1376,7 @@
         <v>24</v>
       </c>
       <c r="B8">
-        <v>1174</v>
+        <v>1222</v>
       </c>
       <c r="C8" t="s">
         <v>65</v>
@@ -1394,16 +1394,16 @@
         <v>1</v>
       </c>
       <c r="H8">
-        <v>577</v>
+        <v>744</v>
       </c>
       <c r="I8">
-        <v>556</v>
+        <v>723</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>565</v>
+        <v>732</v>
       </c>
       <c r="L8">
         <v>0</v>
@@ -1412,7 +1412,7 @@
         <v>162</v>
       </c>
       <c r="N8" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="O8">
         <v>100</v>
@@ -1429,7 +1429,7 @@
         <v>25</v>
       </c>
       <c r="B9">
-        <v>1175</v>
+        <v>1200</v>
       </c>
       <c r="C9" t="s">
         <v>66</v>
@@ -1447,16 +1447,16 @@
         <v>1</v>
       </c>
       <c r="H9">
-        <v>641</v>
+        <v>578</v>
       </c>
       <c r="I9">
-        <v>620</v>
+        <v>557</v>
       </c>
       <c r="J9">
         <v>0</v>
       </c>
       <c r="K9">
-        <v>629</v>
+        <v>566</v>
       </c>
       <c r="L9">
         <v>0</v>
@@ -1485,7 +1485,7 @@
         <v>26</v>
       </c>
       <c r="B10">
-        <v>1210</v>
+        <v>1235</v>
       </c>
       <c r="C10" t="s">
         <v>67</v>
@@ -1521,7 +1521,7 @@
         <v>164</v>
       </c>
       <c r="N10" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="O10">
         <v>100</v>
@@ -1541,7 +1541,7 @@
         <v>27</v>
       </c>
       <c r="B11">
-        <v>1107</v>
+        <v>1210</v>
       </c>
       <c r="C11" t="s">
         <v>68</v>
@@ -1559,16 +1559,16 @@
         <v>1</v>
       </c>
       <c r="H11">
-        <v>577</v>
+        <v>641</v>
       </c>
       <c r="I11">
-        <v>556</v>
+        <v>620</v>
       </c>
       <c r="J11">
         <v>0</v>
       </c>
       <c r="K11">
-        <v>565</v>
+        <v>629</v>
       </c>
       <c r="L11">
         <v>0</v>
@@ -1577,9 +1577,12 @@
         <v>165</v>
       </c>
       <c r="N11" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="O11">
+        <v>100</v>
+      </c>
+      <c r="P11">
         <v>100</v>
       </c>
       <c r="Q11">
@@ -1594,7 +1597,7 @@
         <v>28</v>
       </c>
       <c r="B12">
-        <v>1196</v>
+        <v>1175</v>
       </c>
       <c r="C12" t="s">
         <v>69</v>
@@ -1612,16 +1615,16 @@
         <v>1</v>
       </c>
       <c r="H12">
-        <v>578</v>
+        <v>641</v>
       </c>
       <c r="I12">
-        <v>557</v>
+        <v>620</v>
       </c>
       <c r="J12">
         <v>0</v>
       </c>
       <c r="K12">
-        <v>566</v>
+        <v>629</v>
       </c>
       <c r="L12">
         <v>0</v>
@@ -1630,7 +1633,7 @@
         <v>166</v>
       </c>
       <c r="N12" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="O12">
         <v>100</v>
@@ -1650,16 +1653,16 @@
         <v>29</v>
       </c>
       <c r="B13">
-        <v>1171</v>
+        <v>1110</v>
       </c>
       <c r="C13" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="D13" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="E13" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
       <c r="F13" t="s">
         <v>155</v>
@@ -1668,30 +1671,27 @@
         <v>1</v>
       </c>
       <c r="H13">
-        <v>641</v>
+        <v>577</v>
       </c>
       <c r="I13">
-        <v>620</v>
+        <v>556</v>
       </c>
       <c r="J13">
         <v>0</v>
       </c>
       <c r="K13">
-        <v>629</v>
+        <v>565</v>
       </c>
       <c r="L13">
         <v>0</v>
       </c>
       <c r="M13" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
       <c r="N13" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="O13">
-        <v>100</v>
-      </c>
-      <c r="P13">
         <v>100</v>
       </c>
       <c r="Q13">
@@ -1706,16 +1706,16 @@
         <v>30</v>
       </c>
       <c r="B14">
-        <v>1200</v>
+        <v>1107</v>
       </c>
       <c r="C14" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D14" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E14" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F14" t="s">
         <v>155</v>
@@ -1724,30 +1724,27 @@
         <v>1</v>
       </c>
       <c r="H14">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="I14">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="J14">
         <v>0</v>
       </c>
       <c r="K14">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="L14">
         <v>0</v>
       </c>
       <c r="M14" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="N14" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="O14">
-        <v>100</v>
-      </c>
-      <c r="P14">
         <v>100</v>
       </c>
       <c r="Q14">
@@ -1765,13 +1762,13 @@
         <v>1171</v>
       </c>
       <c r="C15" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D15" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F15" t="s">
         <v>155</v>
@@ -1780,27 +1777,30 @@
         <v>1</v>
       </c>
       <c r="H15">
-        <v>577</v>
+        <v>641</v>
       </c>
       <c r="I15">
-        <v>556</v>
+        <v>620</v>
       </c>
       <c r="J15">
         <v>0</v>
       </c>
       <c r="K15">
-        <v>565</v>
+        <v>629</v>
       </c>
       <c r="L15">
         <v>0</v>
       </c>
       <c r="M15" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="N15" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="O15">
+        <v>100</v>
+      </c>
+      <c r="P15">
         <v>100</v>
       </c>
       <c r="Q15">
@@ -1815,16 +1815,16 @@
         <v>32</v>
       </c>
       <c r="B16">
-        <v>1110</v>
+        <v>1171</v>
       </c>
       <c r="C16" t="s">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="D16" t="s">
-        <v>96</v>
+        <v>104</v>
       </c>
       <c r="E16" t="s">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="F16" t="s">
         <v>155</v>
@@ -1848,7 +1848,7 @@
         <v>0</v>
       </c>
       <c r="M16" t="s">
-        <v>161</v>
+        <v>169</v>
       </c>
       <c r="N16" t="s">
         <v>189</v>
@@ -1868,16 +1868,16 @@
         <v>33</v>
       </c>
       <c r="B17">
-        <v>1170</v>
+        <v>1237</v>
       </c>
       <c r="C17" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="D17" t="s">
-        <v>96</v>
+        <v>105</v>
       </c>
       <c r="E17" t="s">
-        <v>128</v>
+        <v>137</v>
       </c>
       <c r="F17" t="s">
         <v>155</v>
@@ -1886,27 +1886,30 @@
         <v>1</v>
       </c>
       <c r="H17">
-        <v>577</v>
+        <v>641</v>
       </c>
       <c r="I17">
-        <v>556</v>
+        <v>620</v>
       </c>
       <c r="J17">
         <v>0</v>
       </c>
       <c r="K17">
-        <v>565</v>
+        <v>629</v>
       </c>
       <c r="L17">
         <v>0</v>
       </c>
       <c r="M17" t="s">
-        <v>161</v>
+        <v>170</v>
       </c>
       <c r="N17" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="O17">
+        <v>100</v>
+      </c>
+      <c r="P17">
         <v>100</v>
       </c>
       <c r="Q17">
@@ -1921,16 +1924,16 @@
         <v>34</v>
       </c>
       <c r="B18">
-        <v>1237</v>
+        <v>1177</v>
       </c>
       <c r="C18" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="D18" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="E18" t="s">
-        <v>137</v>
+        <v>129</v>
       </c>
       <c r="F18" t="s">
         <v>155</v>
@@ -1939,30 +1942,27 @@
         <v>1</v>
       </c>
       <c r="H18">
-        <v>641</v>
+        <v>744</v>
       </c>
       <c r="I18">
-        <v>620</v>
+        <v>723</v>
       </c>
       <c r="J18">
         <v>0</v>
       </c>
       <c r="K18">
-        <v>629</v>
+        <v>732</v>
       </c>
       <c r="L18">
         <v>0</v>
       </c>
       <c r="M18" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="N18" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="O18">
-        <v>100</v>
-      </c>
-      <c r="P18">
         <v>100</v>
       </c>
       <c r="Q18">
@@ -1977,16 +1977,16 @@
         <v>35</v>
       </c>
       <c r="B19">
-        <v>1177</v>
+        <v>1184</v>
       </c>
       <c r="C19" t="s">
-        <v>62</v>
+        <v>74</v>
       </c>
       <c r="D19" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
       <c r="E19" t="s">
-        <v>126</v>
+        <v>138</v>
       </c>
       <c r="F19" t="s">
         <v>155</v>
@@ -1995,27 +1995,30 @@
         <v>1</v>
       </c>
       <c r="H19">
-        <v>744</v>
+        <v>743</v>
       </c>
       <c r="I19">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="J19">
         <v>0</v>
       </c>
       <c r="K19">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="L19">
         <v>0</v>
       </c>
       <c r="M19" t="s">
-        <v>159</v>
+        <v>171</v>
       </c>
       <c r="N19" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="O19">
+        <v>100</v>
+      </c>
+      <c r="P19">
         <v>100</v>
       </c>
       <c r="Q19">
@@ -2030,16 +2033,16 @@
         <v>36</v>
       </c>
       <c r="B20">
-        <v>1184</v>
+        <v>1170</v>
       </c>
       <c r="C20" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="D20" t="s">
-        <v>106</v>
+        <v>94</v>
       </c>
       <c r="E20" t="s">
-        <v>138</v>
+        <v>126</v>
       </c>
       <c r="F20" t="s">
         <v>155</v>
@@ -2048,30 +2051,27 @@
         <v>1</v>
       </c>
       <c r="H20">
-        <v>743</v>
+        <v>577</v>
       </c>
       <c r="I20">
-        <v>722</v>
+        <v>556</v>
       </c>
       <c r="J20">
         <v>0</v>
       </c>
       <c r="K20">
-        <v>731</v>
+        <v>565</v>
       </c>
       <c r="L20">
         <v>0</v>
       </c>
       <c r="M20" t="s">
-        <v>171</v>
+        <v>159</v>
       </c>
       <c r="N20" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="O20">
-        <v>100</v>
-      </c>
-      <c r="P20">
         <v>100</v>
       </c>
       <c r="Q20">
@@ -2086,7 +2086,7 @@
         <v>37</v>
       </c>
       <c r="B21">
-        <v>1240</v>
+        <v>1174</v>
       </c>
       <c r="C21" t="s">
         <v>75</v>
@@ -2104,16 +2104,16 @@
         <v>1</v>
       </c>
       <c r="H21">
-        <v>742</v>
+        <v>641</v>
       </c>
       <c r="I21">
-        <v>721</v>
+        <v>620</v>
       </c>
       <c r="J21">
         <v>0</v>
       </c>
       <c r="K21">
-        <v>730</v>
+        <v>629</v>
       </c>
       <c r="L21">
         <v>0</v>
@@ -2122,9 +2122,12 @@
         <v>172</v>
       </c>
       <c r="N21" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="O21">
+        <v>100</v>
+      </c>
+      <c r="P21">
         <v>100</v>
       </c>
       <c r="Q21">
@@ -2139,7 +2142,7 @@
         <v>38</v>
       </c>
       <c r="B22">
-        <v>1174</v>
+        <v>1235</v>
       </c>
       <c r="C22" t="s">
         <v>76</v>
@@ -2175,7 +2178,7 @@
         <v>173</v>
       </c>
       <c r="N22" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="O22">
         <v>100</v>
@@ -2195,7 +2198,7 @@
         <v>39</v>
       </c>
       <c r="B23">
-        <v>1074</v>
+        <v>1163</v>
       </c>
       <c r="C23" t="s">
         <v>77</v>
@@ -2210,30 +2213,33 @@
         <v>155</v>
       </c>
       <c r="G23">
-        <v>1</v>
+        <v>0.9987405541561712</v>
       </c>
       <c r="H23">
-        <v>579</v>
+        <v>806</v>
       </c>
       <c r="I23">
-        <v>558</v>
+        <v>783</v>
       </c>
       <c r="J23">
         <v>0</v>
       </c>
       <c r="K23">
-        <v>567</v>
+        <v>794</v>
       </c>
       <c r="L23">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M23" t="s">
         <v>174</v>
       </c>
       <c r="N23" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="O23">
+        <v>99.22480620155039</v>
+      </c>
+      <c r="P23">
         <v>100</v>
       </c>
       <c r="Q23">
@@ -2248,7 +2254,7 @@
         <v>40</v>
       </c>
       <c r="B24">
-        <v>1173</v>
+        <v>1189</v>
       </c>
       <c r="C24" t="s">
         <v>78</v>
@@ -2266,16 +2272,16 @@
         <v>1</v>
       </c>
       <c r="H24">
-        <v>641</v>
+        <v>578</v>
       </c>
       <c r="I24">
-        <v>620</v>
+        <v>557</v>
       </c>
       <c r="J24">
         <v>0</v>
       </c>
       <c r="K24">
-        <v>629</v>
+        <v>566</v>
       </c>
       <c r="L24">
         <v>0</v>
@@ -2304,7 +2310,7 @@
         <v>41</v>
       </c>
       <c r="B25">
-        <v>1235</v>
+        <v>1240</v>
       </c>
       <c r="C25" t="s">
         <v>79</v>
@@ -2322,16 +2328,16 @@
         <v>1</v>
       </c>
       <c r="H25">
-        <v>641</v>
+        <v>742</v>
       </c>
       <c r="I25">
-        <v>620</v>
+        <v>721</v>
       </c>
       <c r="J25">
         <v>0</v>
       </c>
       <c r="K25">
-        <v>629</v>
+        <v>730</v>
       </c>
       <c r="L25">
         <v>0</v>
@@ -2340,12 +2346,9 @@
         <v>176</v>
       </c>
       <c r="N25" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
       <c r="O25">
-        <v>100</v>
-      </c>
-      <c r="P25">
         <v>100</v>
       </c>
       <c r="Q25">
@@ -2413,16 +2416,16 @@
         <v>43</v>
       </c>
       <c r="B27">
-        <v>1230</v>
+        <v>1074</v>
       </c>
       <c r="C27" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="D27" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="E27" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="F27" t="s">
         <v>155</v>
@@ -2431,25 +2434,25 @@
         <v>1</v>
       </c>
       <c r="H27">
-        <v>742</v>
+        <v>579</v>
       </c>
       <c r="I27">
-        <v>721</v>
+        <v>558</v>
       </c>
       <c r="J27">
         <v>0</v>
       </c>
       <c r="K27">
-        <v>730</v>
+        <v>567</v>
       </c>
       <c r="L27">
         <v>0</v>
       </c>
       <c r="M27" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="N27" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="O27">
         <v>100</v>
@@ -2466,45 +2469,48 @@
         <v>44</v>
       </c>
       <c r="B28">
-        <v>1245</v>
+        <v>1228</v>
       </c>
       <c r="C28" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D28" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E28" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="F28" t="s">
         <v>155</v>
       </c>
       <c r="G28">
-        <v>1</v>
+        <v>0.9987405541561712</v>
       </c>
       <c r="H28">
-        <v>579</v>
+        <v>806</v>
       </c>
       <c r="I28">
-        <v>558</v>
+        <v>783</v>
       </c>
       <c r="J28">
         <v>0</v>
       </c>
       <c r="K28">
-        <v>567</v>
+        <v>794</v>
       </c>
       <c r="L28">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M28" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="N28" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="O28">
+        <v>99.73753280839895</v>
+      </c>
+      <c r="P28">
         <v>100</v>
       </c>
       <c r="Q28">
@@ -2519,46 +2525,46 @@
         <v>45</v>
       </c>
       <c r="B29">
-        <v>1163</v>
+        <v>1171</v>
       </c>
       <c r="C29" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D29" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E29" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="F29" t="s">
         <v>155</v>
       </c>
       <c r="G29">
-        <v>0.9987405541561712</v>
+        <v>1</v>
       </c>
       <c r="H29">
-        <v>806</v>
+        <v>641</v>
       </c>
       <c r="I29">
-        <v>783</v>
+        <v>620</v>
       </c>
       <c r="J29">
         <v>0</v>
       </c>
       <c r="K29">
-        <v>794</v>
+        <v>629</v>
       </c>
       <c r="L29">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M29" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="N29" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="O29">
-        <v>99.22480620155039</v>
+        <v>100</v>
       </c>
       <c r="P29">
         <v>100</v>
@@ -2575,16 +2581,16 @@
         <v>46</v>
       </c>
       <c r="B30">
-        <v>1189</v>
+        <v>1245</v>
       </c>
       <c r="C30" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D30" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="E30" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F30" t="s">
         <v>155</v>
@@ -2593,30 +2599,27 @@
         <v>1</v>
       </c>
       <c r="H30">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="I30">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="J30">
         <v>0</v>
       </c>
       <c r="K30">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="L30">
         <v>0</v>
       </c>
       <c r="M30" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="N30" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="O30">
-        <v>100</v>
-      </c>
-      <c r="P30">
         <v>100</v>
       </c>
       <c r="Q30">
@@ -2631,16 +2634,16 @@
         <v>47</v>
       </c>
       <c r="B31">
-        <v>1171</v>
+        <v>1196</v>
       </c>
       <c r="C31" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D31" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E31" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F31" t="s">
         <v>155</v>
@@ -2649,22 +2652,22 @@
         <v>1</v>
       </c>
       <c r="H31">
-        <v>641</v>
+        <v>578</v>
       </c>
       <c r="I31">
-        <v>620</v>
+        <v>557</v>
       </c>
       <c r="J31">
         <v>0</v>
       </c>
       <c r="K31">
-        <v>629</v>
+        <v>566</v>
       </c>
       <c r="L31">
         <v>0</v>
       </c>
       <c r="M31" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="N31" t="s">
         <v>190</v>
@@ -2687,16 +2690,16 @@
         <v>48</v>
       </c>
       <c r="B32">
-        <v>1228</v>
+        <v>1173</v>
       </c>
       <c r="C32" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="D32" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="E32" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="F32" t="s">
         <v>155</v>
@@ -2705,25 +2708,25 @@
         <v>1</v>
       </c>
       <c r="H32">
-        <v>806</v>
+        <v>641</v>
       </c>
       <c r="I32">
-        <v>785</v>
+        <v>620</v>
       </c>
       <c r="J32">
         <v>0</v>
       </c>
       <c r="K32">
-        <v>794</v>
+        <v>629</v>
       </c>
       <c r="L32">
         <v>0</v>
       </c>
       <c r="M32" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="N32" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="O32">
         <v>100</v>
@@ -2743,16 +2746,16 @@
         <v>49</v>
       </c>
       <c r="B33">
-        <v>1185</v>
+        <v>1230</v>
       </c>
       <c r="C33" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="D33" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="E33" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="F33" t="s">
         <v>155</v>
@@ -2761,30 +2764,27 @@
         <v>1</v>
       </c>
       <c r="H33">
-        <v>578</v>
+        <v>742</v>
       </c>
       <c r="I33">
-        <v>557</v>
+        <v>721</v>
       </c>
       <c r="J33">
         <v>0</v>
       </c>
       <c r="K33">
-        <v>566</v>
+        <v>730</v>
       </c>
       <c r="L33">
         <v>0</v>
       </c>
       <c r="M33" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="N33" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="O33">
-        <v>100</v>
-      </c>
-      <c r="P33">
         <v>100</v>
       </c>
       <c r="Q33">
@@ -2799,16 +2799,16 @@
         <v>50</v>
       </c>
       <c r="B34">
-        <v>1196</v>
+        <v>1193</v>
       </c>
       <c r="C34" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D34" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E34" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="F34" t="s">
         <v>155</v>
@@ -2835,7 +2835,7 @@
         <v>183</v>
       </c>
       <c r="N34" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="O34">
         <v>100</v>
@@ -2858,25 +2858,25 @@
         <v>1228</v>
       </c>
       <c r="C35" t="s">
-        <v>86</v>
+        <v>77</v>
       </c>
       <c r="D35" t="s">
-        <v>118</v>
+        <v>109</v>
       </c>
       <c r="E35" t="s">
-        <v>150</v>
+        <v>141</v>
       </c>
       <c r="F35" t="s">
         <v>155</v>
       </c>
       <c r="G35">
-        <v>0.9987405541561712</v>
+        <v>1</v>
       </c>
       <c r="H35">
         <v>806</v>
       </c>
       <c r="I35">
-        <v>783</v>
+        <v>785</v>
       </c>
       <c r="J35">
         <v>0</v>
@@ -2885,16 +2885,16 @@
         <v>794</v>
       </c>
       <c r="L35">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M35" t="s">
         <v>184</v>
       </c>
       <c r="N35" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="O35">
-        <v>99.73753280839895</v>
+        <v>100</v>
       </c>
       <c r="P35">
         <v>100</v>
@@ -2911,16 +2911,16 @@
         <v>52</v>
       </c>
       <c r="B36">
-        <v>1242</v>
+        <v>1240</v>
       </c>
       <c r="C36" t="s">
-        <v>87</v>
+        <v>59</v>
       </c>
       <c r="D36" t="s">
-        <v>119</v>
+        <v>91</v>
       </c>
       <c r="E36" t="s">
-        <v>151</v>
+        <v>123</v>
       </c>
       <c r="F36" t="s">
         <v>155</v>
@@ -2944,7 +2944,7 @@
         <v>0</v>
       </c>
       <c r="M36" t="s">
-        <v>185</v>
+        <v>156</v>
       </c>
       <c r="N36" t="s">
         <v>189</v>
@@ -2964,16 +2964,16 @@
         <v>53</v>
       </c>
       <c r="B37">
-        <v>1244</v>
+        <v>1191</v>
       </c>
       <c r="C37" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D37" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E37" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F37" t="s">
         <v>155</v>
@@ -2982,27 +2982,30 @@
         <v>1</v>
       </c>
       <c r="H37">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="I37">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="J37">
         <v>0</v>
       </c>
       <c r="K37">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="L37">
         <v>0</v>
       </c>
       <c r="M37" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="N37" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
       <c r="O37">
+        <v>100</v>
+      </c>
+      <c r="P37">
         <v>100</v>
       </c>
       <c r="Q37">
@@ -3017,16 +3020,16 @@
         <v>54</v>
       </c>
       <c r="B38">
-        <v>1193</v>
+        <v>1203</v>
       </c>
       <c r="C38" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D38" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E38" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="F38" t="s">
         <v>155</v>
@@ -3035,30 +3038,27 @@
         <v>1</v>
       </c>
       <c r="H38">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="I38">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="J38">
         <v>0</v>
       </c>
       <c r="K38">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="L38">
         <v>0</v>
       </c>
       <c r="M38" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="N38" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="O38">
-        <v>100</v>
-      </c>
-      <c r="P38">
         <v>100</v>
       </c>
       <c r="Q38">
@@ -3073,16 +3073,16 @@
         <v>55</v>
       </c>
       <c r="B39">
-        <v>1240</v>
+        <v>1185</v>
       </c>
       <c r="C39" t="s">
-        <v>59</v>
+        <v>87</v>
       </c>
       <c r="D39" t="s">
-        <v>91</v>
+        <v>119</v>
       </c>
       <c r="E39" t="s">
-        <v>123</v>
+        <v>151</v>
       </c>
       <c r="F39" t="s">
         <v>155</v>
@@ -3091,27 +3091,30 @@
         <v>1</v>
       </c>
       <c r="H39">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="I39">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="J39">
         <v>0</v>
       </c>
       <c r="K39">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="L39">
         <v>0</v>
       </c>
       <c r="M39" t="s">
-        <v>156</v>
+        <v>185</v>
       </c>
       <c r="N39" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="O39">
+        <v>100</v>
+      </c>
+      <c r="P39">
         <v>100</v>
       </c>
       <c r="Q39">
@@ -3126,16 +3129,16 @@
         <v>56</v>
       </c>
       <c r="B40">
-        <v>1203</v>
+        <v>1201</v>
       </c>
       <c r="C40" t="s">
-        <v>90</v>
+        <v>61</v>
       </c>
       <c r="D40" t="s">
-        <v>122</v>
+        <v>93</v>
       </c>
       <c r="E40" t="s">
-        <v>154</v>
+        <v>125</v>
       </c>
       <c r="F40" t="s">
         <v>155</v>
@@ -3144,25 +3147,25 @@
         <v>1</v>
       </c>
       <c r="H40">
-        <v>579</v>
+        <v>577</v>
       </c>
       <c r="I40">
-        <v>558</v>
+        <v>556</v>
       </c>
       <c r="J40">
         <v>0</v>
       </c>
       <c r="K40">
-        <v>567</v>
+        <v>565</v>
       </c>
       <c r="L40">
         <v>0</v>
       </c>
       <c r="M40" t="s">
-        <v>188</v>
+        <v>158</v>
       </c>
       <c r="N40" t="s">
-        <v>195</v>
+        <v>189</v>
       </c>
       <c r="O40">
         <v>100</v>
@@ -3179,16 +3182,16 @@
         <v>57</v>
       </c>
       <c r="B41">
-        <v>1201</v>
+        <v>1244</v>
       </c>
       <c r="C41" t="s">
-        <v>65</v>
+        <v>89</v>
       </c>
       <c r="D41" t="s">
-        <v>97</v>
+        <v>121</v>
       </c>
       <c r="E41" t="s">
-        <v>129</v>
+        <v>153</v>
       </c>
       <c r="F41" t="s">
         <v>155</v>
@@ -3197,25 +3200,25 @@
         <v>1</v>
       </c>
       <c r="H41">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="I41">
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="J41">
         <v>0</v>
       </c>
       <c r="K41">
-        <v>565</v>
+        <v>567</v>
       </c>
       <c r="L41">
         <v>0</v>
       </c>
       <c r="M41" t="s">
-        <v>162</v>
+        <v>187</v>
       </c>
       <c r="N41" t="s">
-        <v>189</v>
+        <v>196</v>
       </c>
       <c r="O41">
         <v>100</v>
@@ -3232,16 +3235,16 @@
         <v>58</v>
       </c>
       <c r="B42">
-        <v>1191</v>
+        <v>1242</v>
       </c>
       <c r="C42" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="D42" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="E42" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="F42" t="s">
         <v>155</v>
@@ -3250,30 +3253,27 @@
         <v>1</v>
       </c>
       <c r="H42">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="I42">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="J42">
         <v>0</v>
       </c>
       <c r="K42">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="L42">
         <v>0</v>
       </c>
       <c r="M42" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="N42" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="O42">
-        <v>100</v>
-      </c>
-      <c r="P42">
         <v>100</v>
       </c>
       <c r="Q42">

</xml_diff>